<commit_message>
Ajusta processamento de e-mails e anexos nos relatórios
Atualiza o script de processamento de erros para capturar apenas e-mails do dia atual e adiciona tratamento de exceção ao carregar arquivos Excel. Corrige a lógica de anexos no envio de relatórios para empresas do grupo Kontik. Atualiza diversos arquivos Excel e adiciona novos relatórios PDF para 12.08.2025 e 13.08.2025.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - ZUPPER VIAGENS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - ZUPPER VIAGENS.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ6"/>
+  <dimension ref="A1:AQ5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,21 +695,21 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>22701701</v>
+        <v>22730377</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>23503867</v>
+        <v>23527875</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>45876.65152777778</v>
+        <v>45881.6105787037</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>45876.6568287037</v>
+        <v>45881.61115740741</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
@@ -723,36 +723,34 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>ZWHCTQ</t>
+          <t>AYSZPQ</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>ANA CARVALHO</t>
+          <t>Jaqueline Bonino</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Laura Sales de Paula</t>
+          <t>Zupper</t>
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>Laura Sales de Paula</t>
+          <t>Zupper</t>
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>45875.65138888889</v>
-      </c>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>45881.60972222222</v>
+      </c>
+      <c r="N2" s="5" t="n">
+        <v>6807340</v>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
@@ -801,11 +799,11 @@
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y2" s="5" t="n">
-        <v>3023503866</v>
+        <v>2143299117</v>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
@@ -818,16 +816,16 @@
         </is>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>708.9</v>
+        <v>522.9</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>46.36</v>
+        <v>33.64</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE2" s="5" t="n">
-        <v>0</v>
+        <v>52.29</v>
       </c>
       <c r="AF2" s="5" t="n">
         <v>0</v>
@@ -836,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>56.71</v>
+        <v>0</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
@@ -845,7 +843,7 @@
       </c>
       <c r="AJ2" s="5" t="inlineStr">
         <is>
-          <t>36Faltou informar rateio de centro de custo/projeto abaixo da accounting</t>
+          <t>Pnr já existente. A duplicidade de rloc é permitida apenas 6 meses após o último pnr emitido</t>
         </is>
       </c>
       <c r="AK2" s="5" t="inlineStr">
@@ -855,17 +853,17 @@
       </c>
       <c r="AL2" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Duplicidade de RLOC</t>
         </is>
       </c>
       <c r="AM2" s="5" t="inlineStr">
         <is>
-          <t>Rateio de centro de custo/projeto</t>
+          <t>Campo RLOC</t>
         </is>
       </c>
       <c r="AN2" s="5" t="inlineStr">
         <is>
-          <t>Dados Gerenciais</t>
+          <t>Duplicidade de Contabilização</t>
         </is>
       </c>
       <c r="AO2" s="5" t="inlineStr">
@@ -886,10 +884,10 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>22701543</v>
+        <v>22734093</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>23503696</v>
+        <v>23531368</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -897,10 +895,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>45876.62931712963</v>
+        <v>45882.0294212963</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>45876.64641203704</v>
+        <v>45882.03172453704</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -914,7 +912,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>XEE5VR</t>
+          <t>QHEFPA</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -924,7 +922,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>CARLOS EDUARDO OLIVEIRA SA</t>
+          <t>Hannah Assayag</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -938,10 +936,10 @@
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>45876.62847222222</v>
+        <v>45882.02847222222</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>6800303</v>
+        <v>6808127</v>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -955,12 +953,12 @@
       </c>
       <c r="Q3" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R3" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão convênio</t>
         </is>
       </c>
       <c r="S3" s="5" t="inlineStr">
@@ -980,7 +978,7 @@
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>Carlos e O Sa</t>
+          <t>Cristiani Oliveira</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
@@ -990,11 +988,11 @@
       </c>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>6359382136</v>
+        <v>2245618947</v>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
@@ -1007,10 +1005,10 @@
         </is>
       </c>
       <c r="AB3" s="5" t="n">
-        <v>1249.37</v>
+        <v>444.72</v>
       </c>
       <c r="AC3" s="5" t="n">
-        <v>106.98</v>
+        <v>33.64</v>
       </c>
       <c r="AD3" s="5" t="n">
         <v>0</v>
@@ -1025,7 +1023,7 @@
         <v>0</v>
       </c>
       <c r="AH3" s="5" t="n">
-        <v>224.88</v>
+        <v>64.04000000000001</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
@@ -1034,7 +1032,7 @@
       </c>
       <c r="AJ3" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 07/08/2025</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 2 e Data transação 13/08/2025</t>
         </is>
       </c>
       <c r="AK3" s="5" t="inlineStr">
@@ -1075,21 +1073,21 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>22701543</v>
+        <v>22734114</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>23503698</v>
+        <v>23531379</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>45876.62931712963</v>
+        <v>45882.03140046296</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>45876.64641203704</v>
+        <v>45882.03368055556</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -1103,7 +1101,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>XEE5VR</t>
+          <t>BNYPQA</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -1113,7 +1111,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>CATARINA FATIMA OLIVEIRA</t>
+          <t>Nubia Silva</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1127,10 +1125,10 @@
         </is>
       </c>
       <c r="M4" s="6" t="n">
-        <v>45876.62847222222</v>
+        <v>45882.03055555555</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>6800303</v>
+        <v>6808139</v>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
@@ -1144,12 +1142,12 @@
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão convênio</t>
         </is>
       </c>
       <c r="S4" s="5" t="inlineStr">
@@ -1169,7 +1167,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>Carlos e O Sa</t>
+          <t>Nubia Erica m da silva</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1183,7 +1181,7 @@
         </is>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>5083348355</v>
+        <v>183917540</v>
       </c>
       <c r="Z4" s="5" t="inlineStr">
         <is>
@@ -1196,10 +1194,10 @@
         </is>
       </c>
       <c r="AB4" s="5" t="n">
-        <v>1249.37</v>
+        <v>1032.3</v>
       </c>
       <c r="AC4" s="5" t="n">
-        <v>106.98</v>
+        <v>58.89</v>
       </c>
       <c r="AD4" s="5" t="n">
         <v>0</v>
@@ -1214,7 +1212,7 @@
         <v>0</v>
       </c>
       <c r="AH4" s="5" t="n">
-        <v>0</v>
+        <v>147.27</v>
       </c>
       <c r="AI4" s="5" t="inlineStr">
         <is>
@@ -1223,7 +1221,7 @@
       </c>
       <c r="AJ4" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data Emissão 07/08/2025</t>
+          <t>Não foi possível encontrar configuração válida para Administradora de código 1 e Data transação 13/08/2025</t>
         </is>
       </c>
       <c r="AK4" s="5" t="inlineStr">
@@ -1264,10 +1262,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>22705296</v>
+        <v>22733433</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>23507214</v>
+        <v>23530759</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -1275,10 +1273,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>45877.04255787037</v>
+        <v>45881.94744212963</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>45877.04537037037</v>
+        <v>45881.94872685185</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -1292,7 +1290,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>XQUV5U</t>
+          <t>MKCKTB</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -1302,7 +1300,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>RAIMUNDA JULIA BRANDAO</t>
+          <t>Luciene Oliveira</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1316,10 +1314,10 @@
         </is>
       </c>
       <c r="M5" s="6" t="n">
-        <v>45877.04097222222</v>
+        <v>45881.94652777778</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>6802172</v>
+        <v>6807991</v>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
@@ -1333,12 +1331,12 @@
       </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão convênio</t>
         </is>
       </c>
       <c r="S5" s="5" t="inlineStr">
@@ -1358,7 +1356,7 @@
       </c>
       <c r="V5" s="5" t="inlineStr">
         <is>
-          <t>Raimunda Julia de Freitas Brandao</t>
+          <t>Luciene Costa de Oliveira</t>
         </is>
       </c>
       <c r="W5" s="5" t="inlineStr">
@@ -1368,11 +1366,11 @@
       </c>
       <c r="X5" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>8282448174</v>
+        <v>2245603129</v>
       </c>
       <c r="Z5" s="5" t="inlineStr">
         <is>
@@ -1385,10 +1383,10 @@
         </is>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>361.68</v>
+        <v>848.64</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>54.45</v>
+        <v>92.53</v>
       </c>
       <c r="AD5" s="5" t="n">
         <v>0</v>
@@ -1403,7 +1401,7 @@
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="n">
-        <v>32.55</v>
+        <v>122.2</v>
       </c>
       <c r="AI5" s="5" t="inlineStr">
         <is>
@@ -1446,197 +1444,6 @@
         </is>
       </c>
       <c r="AQ5" s="5" t="inlineStr">
-        <is>
-          <t>Operações - ZUPPER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>22703334</v>
-      </c>
-      <c r="B6" s="5" t="n">
-        <v>23505442</v>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>ACC01</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>45876.78077546296</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>45876.80650462963</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>0 a 02 dias</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>0 a 02 dias</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>5GCXYC</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>TMS</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>CARLOS OLIVEIRA</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>Tms</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>Tms</t>
-        </is>
-      </c>
-      <c r="M6" s="6" t="n">
-        <v>45876.53055555555</v>
-      </c>
-      <c r="N6" s="5" t="n">
-        <v>386</v>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Taubate / QHP</t>
-        </is>
-      </c>
-      <c r="P6" s="5" t="inlineStr">
-        <is>
-          <t>ON LINE</t>
-        </is>
-      </c>
-      <c r="Q6" s="5" t="inlineStr">
-        <is>
-          <t>Invoice</t>
-        </is>
-      </c>
-      <c r="R6" s="5" t="inlineStr">
-        <is>
-          <t>Faturado</t>
-        </is>
-      </c>
-      <c r="S6" s="5" t="inlineStr">
-        <is>
-          <t>Carro</t>
-        </is>
-      </c>
-      <c r="T6" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="U6" s="5" t="inlineStr">
-        <is>
-          <t>Grupo Zupper</t>
-        </is>
-      </c>
-      <c r="V6" s="5" t="inlineStr">
-        <is>
-          <t>Zupper Viagens Internas</t>
-        </is>
-      </c>
-      <c r="W6" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X6" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y6" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z6" s="5" t="inlineStr">
-        <is>
-          <t>KON-OPE-SAO-SUP-KONTIK DESPESAS</t>
-        </is>
-      </c>
-      <c r="AA6" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB6" s="5" t="n">
-        <v>537.6900000000001</v>
-      </c>
-      <c r="AC6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI6" s="5" t="inlineStr">
-        <is>
-          <t>Reserva importada do Sistema TMS. OS: 386</t>
-        </is>
-      </c>
-      <c r="AJ6" s="5" t="inlineStr">
-        <is>
-          <t>Fornecedor não preenchido! (ACC01)</t>
-        </is>
-      </c>
-      <c r="AK6" s="5" t="inlineStr">
-        <is>
-          <t>ZUPPER</t>
-        </is>
-      </c>
-      <c r="AL6" s="5" t="inlineStr">
-        <is>
-          <t>Falta de Fornecedor</t>
-        </is>
-      </c>
-      <c r="AM6" s="5" t="inlineStr">
-        <is>
-          <t>Campo Fornecedor</t>
-        </is>
-      </c>
-      <c r="AN6" s="5" t="inlineStr">
-        <is>
-          <t>Dados do Fornecedor</t>
-        </is>
-      </c>
-      <c r="AO6" s="5" t="inlineStr">
-        <is>
-          <t>Qualidade dos dados</t>
-        </is>
-      </c>
-      <c r="AP6" s="5" t="inlineStr">
-        <is>
-          <t>ZUPPER VIAGENS</t>
-        </is>
-      </c>
-      <c r="AQ6" s="5" t="inlineStr">
         <is>
           <t>Operações - ZUPPER</t>
         </is>

</xml_diff>

<commit_message>
Update report files and email logic
Updated several Excel report files with new data. Modified email recipient lists and attachment logic in 4-envio_relatorios.py, including removal of some addresses and disabling attachments for 'Quero Passagem' and 'Integratour' reports. Also removed a script from the execution list in 0-Control_Integration_Quality.py.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - ZUPPER VIAGENS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - ZUPPER VIAGENS.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ14"/>
+  <dimension ref="A1:AQ24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,10 +695,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>23080282</v>
+        <v>23378056</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>23831633</v>
+        <v>24101850</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
@@ -706,10 +706,10 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>45939.75219907407</v>
+        <v>45985.3716087963</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>45939.75254629629</v>
+        <v>45985.37324074074</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>WW2GND</t>
+          <t>UICKQU</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Ricardo Nogueira</t>
+          <t>MARIA CLAUDIA PINHEIRO</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -747,10 +747,10 @@
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>45939.75208333333</v>
+        <v>45985.37083333333</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>6874024</v>
+        <v>6976871</v>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
@@ -764,12 +764,12 @@
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
         <is>
-          <t>Cartão convênio</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>Ricardo Nogueira da Rocha Raimundo</t>
+          <t>Maria Claudia Costa Paunovic</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -799,11 +799,11 @@
       </c>
       <c r="X2" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y2" s="5" t="n">
-        <v>8336454643</v>
+        <v>2150095851</v>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
@@ -816,10 +816,10 @@
         </is>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>2128.2</v>
+        <v>448.73</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>89.75</v>
+        <v>56.88</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>0</v>
+        <v>44.87</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
@@ -884,10 +884,10 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>23077018</v>
+        <v>23379736</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>23828438</v>
+        <v>24103425</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -895,10 +895,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>45939.41193287037</v>
+        <v>45985.63831018518</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>45939.41314814815</v>
+        <v>45985.63976851852</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -912,7 +912,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>YCPIHP</t>
+          <t>NFJUSP</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Ricardo Nogueira</t>
+          <t>Julio Cesar Silva Junior</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -936,10 +936,10 @@
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>45939.41180555556</v>
+        <v>45985.6375</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>6873987</v>
+        <v>6977313</v>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -973,12 +973,12 @@
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Grupo Zupper</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>Ricardo Nogueira da Rocha Raimundo</t>
+          <t>Priscila Cortez Braga Silva</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>4314972148</v>
+        <v>2261090024</v>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
@@ -1005,16 +1005,16 @@
         </is>
       </c>
       <c r="AB3" s="5" t="n">
-        <v>826.08</v>
+        <v>769.52</v>
       </c>
       <c r="AC3" s="5" t="n">
-        <v>86.36</v>
+        <v>56.78</v>
       </c>
       <c r="AD3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE3" s="5" t="n">
-        <v>82.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="AF3" s="5" t="n">
         <v>0</v>
@@ -1023,7 +1023,7 @@
         <v>0</v>
       </c>
       <c r="AH3" s="5" t="n">
-        <v>0</v>
+        <v>230.86</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="AJ3" s="5" t="inlineStr">
         <is>
-          <t>Necessário cadastrar um contrato para o cliente ""</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK3" s="5" t="inlineStr">
@@ -1042,22 +1042,22 @@
       </c>
       <c r="AL3" s="5" t="inlineStr">
         <is>
-          <t>Contrato de fornecedor</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM3" s="5" t="inlineStr">
         <is>
-          <t>Análise Cadastro</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN3" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO3" s="5" t="inlineStr">
         <is>
-          <t>Qualidade dos dados</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP3" s="5" t="inlineStr">
@@ -1073,10 +1073,10 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>23077550</v>
+        <v>23329909</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>23828934</v>
+        <v>24059067</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -1084,32 +1084,34 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>45939.48310185185</v>
+        <v>45976.2847800926</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>45939.48675925926</v>
+        <v>45979.37612268519</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>14229563</v>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>CFLRJQ</t>
+        </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>ANDERSON REIS PEREIRA</t>
+          <t>Rosenir Silva Braga</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1123,12 +1125,10 @@
         </is>
       </c>
       <c r="M4" s="6" t="n">
-        <v>45938.41666666666</v>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>45976.28402777778</v>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>6951692</v>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
@@ -1152,12 +1152,12 @@
       </c>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>Serviço</t>
+          <t>Aéreo</t>
         </is>
       </c>
       <c r="T4" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U4" s="5" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>Anderson Reis Pereira</t>
+          <t>Zupper Cartao</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1177,13 +1177,11 @@
       </c>
       <c r="X4" s="5" t="inlineStr">
         <is>
-          <t>Universal Assistance</t>
-        </is>
-      </c>
-      <c r="Y4" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y4" s="5" t="n">
+        <v>2259793070</v>
       </c>
       <c r="Z4" s="5" t="inlineStr">
         <is>
@@ -1196,10 +1194,10 @@
         </is>
       </c>
       <c r="AB4" s="5" t="n">
-        <v>40.5</v>
+        <v>577.52</v>
       </c>
       <c r="AC4" s="5" t="n">
-        <v>0</v>
+        <v>55.17</v>
       </c>
       <c r="AD4" s="5" t="n">
         <v>0</v>
@@ -1214,16 +1212,16 @@
         <v>0</v>
       </c>
       <c r="AH4" s="5" t="n">
-        <v>0</v>
+        <v>490.9</v>
       </c>
       <c r="AI4" s="5" t="inlineStr">
         <is>
-          <t>Seguro Viagem</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ4" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível definir o Local de destino!</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK4" s="5" t="inlineStr">
@@ -1233,22 +1231,22 @@
       </c>
       <c r="AL4" s="5" t="inlineStr">
         <is>
-          <t>Cadastro enviado errado no Benner</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM4" s="5" t="inlineStr">
         <is>
-          <t>Cadastro incompleto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN4" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO4" s="5" t="inlineStr">
         <is>
-          <t>Sistêmico</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP4" s="5" t="inlineStr">
@@ -1264,43 +1262,45 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>23077510</v>
+        <v>23329909</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>23828901</v>
+        <v>24059068</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>ACC01</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>45939.47814814815</v>
+        <v>45976.2847800926</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>45939.4805787037</v>
+        <v>45979.37612268519</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>14229994</v>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>CFLRJQ</t>
+        </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>RICARDO PINHEIRO</t>
+          <t>Girleno Menezes Barbosa</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1314,12 +1314,10 @@
         </is>
       </c>
       <c r="M5" s="6" t="n">
-        <v>45938.41666666666</v>
-      </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>45976.28402777778</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>6951692</v>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
@@ -1343,12 +1341,12 @@
       </c>
       <c r="S5" s="5" t="inlineStr">
         <is>
-          <t>Serviço</t>
+          <t>Aéreo</t>
         </is>
       </c>
       <c r="T5" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U5" s="5" t="inlineStr">
@@ -1358,7 +1356,7 @@
       </c>
       <c r="V5" s="5" t="inlineStr">
         <is>
-          <t>Ricardo Andre Tiago Pinheiro</t>
+          <t>Zupper Cartao</t>
         </is>
       </c>
       <c r="W5" s="5" t="inlineStr">
@@ -1368,13 +1366,11 @@
       </c>
       <c r="X5" s="5" t="inlineStr">
         <is>
-          <t>Universal Assistance</t>
-        </is>
-      </c>
-      <c r="Y5" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y5" s="5" t="n">
+        <v>2259793071</v>
       </c>
       <c r="Z5" s="5" t="inlineStr">
         <is>
@@ -1387,10 +1383,10 @@
         </is>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>40.5</v>
+        <v>577.52</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>0</v>
+        <v>55.17</v>
       </c>
       <c r="AD5" s="5" t="n">
         <v>0</v>
@@ -1409,12 +1405,12 @@
       </c>
       <c r="AI5" s="5" t="inlineStr">
         <is>
-          <t>Seguro Viagem</t>
+          <t>-</t>
         </is>
       </c>
       <c r="AJ5" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível definir o Local de destino!</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK5" s="5" t="inlineStr">
@@ -1424,22 +1420,22 @@
       </c>
       <c r="AL5" s="5" t="inlineStr">
         <is>
-          <t>Cadastro enviado errado no Benner</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM5" s="5" t="inlineStr">
         <is>
-          <t>Cadastro incompleto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN5" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO5" s="5" t="inlineStr">
         <is>
-          <t>Sistêmico</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP5" s="5" t="inlineStr">
@@ -1455,10 +1451,10 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>23077717</v>
+        <v>23332722</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>23829100</v>
+        <v>24061614</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -1466,24 +1462,24 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>45939.51133101852</v>
+        <v>45976.91744212963</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>45939.51309027777</v>
+        <v>45979.37971064815</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>JAPNDL</t>
+          <t>RLZEGZ</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -1493,7 +1489,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>Maria Gilvaney Cordeiro Lima</t>
+          <t>ADEMIR VALERIO</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1507,10 +1503,10 @@
         </is>
       </c>
       <c r="M6" s="6" t="n">
-        <v>45939.51041666666</v>
+        <v>45976.91666666666</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>6874172</v>
+        <v>6952979</v>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
@@ -1524,12 +1520,12 @@
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão convênio</t>
         </is>
       </c>
       <c r="S6" s="5" t="inlineStr">
@@ -1549,7 +1545,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>Maria Gilvaney Cordeiro Lima</t>
+          <t>Fabiana Sambini</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1559,11 +1555,11 @@
       </c>
       <c r="X6" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Azul Linhas Aereas</t>
         </is>
       </c>
       <c r="Y6" s="5" t="n">
-        <v>2254216553</v>
+        <v>3895134748</v>
       </c>
       <c r="Z6" s="5" t="inlineStr">
         <is>
@@ -1576,16 +1572,16 @@
         </is>
       </c>
       <c r="AB6" s="5" t="n">
-        <v>1139.16</v>
+        <v>1682.08</v>
       </c>
       <c r="AC6" s="5" t="n">
-        <v>59.46</v>
+        <v>92.53</v>
       </c>
       <c r="AD6" s="5" t="n">
         <v>0</v>
       </c>
       <c r="AE6" s="5" t="n">
-        <v>113.91</v>
+        <v>0</v>
       </c>
       <c r="AF6" s="5" t="n">
         <v>0</v>
@@ -1603,7 +1599,7 @@
       </c>
       <c r="AJ6" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível definir o Local de destino!</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25393682. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK6" s="5" t="inlineStr">
@@ -1613,22 +1609,22 @@
       </c>
       <c r="AL6" s="5" t="inlineStr">
         <is>
-          <t>Cadastro enviado errado no Benner</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM6" s="5" t="inlineStr">
         <is>
-          <t>Cadastro incompleto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN6" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO6" s="5" t="inlineStr">
         <is>
-          <t>Sistêmico</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP6" s="5" t="inlineStr">
@@ -1644,10 +1640,10 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>23082254</v>
+        <v>23333521</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>23833470</v>
+        <v>24062221</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -1655,24 +1651,24 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>45939.90564814815</v>
+        <v>45977.14121527778</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>45939.90693287037</v>
+        <v>45979.38116898148</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>IP8YJK</t>
+          <t>WFYUWK</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1682,7 +1678,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>ANTONIO ERINALDO SILVA MARTINS</t>
+          <t>Victoria Cruz</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1696,10 +1692,10 @@
         </is>
       </c>
       <c r="M7" s="6" t="n">
-        <v>45939.90486111111</v>
+        <v>45977.14027777778</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>6874856</v>
+        <v>6953294</v>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
@@ -1713,12 +1709,12 @@
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão convênio</t>
         </is>
       </c>
       <c r="S7" s="5" t="inlineStr">
@@ -1728,7 +1724,7 @@
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
@@ -1738,7 +1734,7 @@
       </c>
       <c r="V7" s="5" t="inlineStr">
         <is>
-          <t>Glauto da Costa Marques</t>
+          <t>Zupper Cartao</t>
         </is>
       </c>
       <c r="W7" s="5" t="inlineStr">
@@ -1748,11 +1744,11 @@
       </c>
       <c r="X7" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>9271566392</v>
+        <v>2259897267</v>
       </c>
       <c r="Z7" s="5" t="inlineStr">
         <is>
@@ -1765,10 +1761,10 @@
         </is>
       </c>
       <c r="AB7" s="5" t="n">
-        <v>245.92</v>
+        <v>1052.72</v>
       </c>
       <c r="AC7" s="5" t="n">
-        <v>33.64</v>
+        <v>56.78</v>
       </c>
       <c r="AD7" s="5" t="n">
         <v>0</v>
@@ -1783,7 +1779,7 @@
         <v>0</v>
       </c>
       <c r="AH7" s="5" t="n">
-        <v>40</v>
+        <v>357.92</v>
       </c>
       <c r="AI7" s="5" t="inlineStr">
         <is>
@@ -1792,7 +1788,7 @@
       </c>
       <c r="AJ7" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível definir o Local de destino!</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25394052. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK7" s="5" t="inlineStr">
@@ -1802,22 +1798,22 @@
       </c>
       <c r="AL7" s="5" t="inlineStr">
         <is>
-          <t>Cadastro enviado errado no Benner</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM7" s="5" t="inlineStr">
         <is>
-          <t>Cadastro incompleto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN7" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO7" s="5" t="inlineStr">
         <is>
-          <t>Sistêmico</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP7" s="5" t="inlineStr">
@@ -1833,10 +1829,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>23082254</v>
+        <v>23333521</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>23833471</v>
+        <v>24062222</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -1844,24 +1840,24 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>45939.90564814815</v>
+        <v>45977.14121527778</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>45939.90693287037</v>
+        <v>45979.38116898148</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>IP8YJK</t>
+          <t>WFYUWK</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1871,7 +1867,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>GLAUTO COSTA MARQUES</t>
+          <t>Benicio Oliveira</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1885,10 +1881,10 @@
         </is>
       </c>
       <c r="M8" s="6" t="n">
-        <v>45939.90486111111</v>
+        <v>45977.14027777778</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>6874856</v>
+        <v>6953294</v>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
@@ -1902,12 +1898,12 @@
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão convênio</t>
         </is>
       </c>
       <c r="S8" s="5" t="inlineStr">
@@ -1917,7 +1913,7 @@
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U8" s="5" t="inlineStr">
@@ -1927,7 +1923,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>Glauto da Costa Marques</t>
+          <t>Zupper Cartao</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1937,11 +1933,11 @@
       </c>
       <c r="X8" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y8" s="5" t="n">
-        <v>4231152706</v>
+        <v>2259897268</v>
       </c>
       <c r="Z8" s="5" t="inlineStr">
         <is>
@@ -1954,10 +1950,10 @@
         </is>
       </c>
       <c r="AB8" s="5" t="n">
-        <v>245.92</v>
+        <v>1052.72</v>
       </c>
       <c r="AC8" s="5" t="n">
-        <v>33.64</v>
+        <v>56.78</v>
       </c>
       <c r="AD8" s="5" t="n">
         <v>0</v>
@@ -1981,7 +1977,7 @@
       </c>
       <c r="AJ8" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível definir o Local de destino!</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25394052. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK8" s="5" t="inlineStr">
@@ -1991,22 +1987,22 @@
       </c>
       <c r="AL8" s="5" t="inlineStr">
         <is>
-          <t>Cadastro enviado errado no Benner</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM8" s="5" t="inlineStr">
         <is>
-          <t>Cadastro incompleto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN8" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO8" s="5" t="inlineStr">
         <is>
-          <t>Sistêmico</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP8" s="5" t="inlineStr">
@@ -2022,35 +2018,35 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>23082254</v>
+        <v>23336052</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>23833472</v>
+        <v>24064344</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>ACC03</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>45939.90564814815</v>
+        <v>45977.7834375</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>45939.90693287037</v>
+        <v>45979.38715277778</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>IP8YJK</t>
+          <t>BL8JGG</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -2060,7 +2056,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>ALEXANDRE MANOEL COSTEIRA NETO</t>
+          <t>Giulianna Delgado</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -2074,10 +2070,10 @@
         </is>
       </c>
       <c r="M9" s="6" t="n">
-        <v>45939.90486111111</v>
+        <v>45977.78263888889</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>6874856</v>
+        <v>6954301</v>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
@@ -2091,12 +2087,12 @@
       </c>
       <c r="Q9" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão convênio</t>
         </is>
       </c>
       <c r="S9" s="5" t="inlineStr">
@@ -2106,7 +2102,7 @@
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U9" s="5" t="inlineStr">
@@ -2116,7 +2112,7 @@
       </c>
       <c r="V9" s="5" t="inlineStr">
         <is>
-          <t>Glauto da Costa Marques</t>
+          <t>Giulianna Angelica Piason de Brito</t>
         </is>
       </c>
       <c r="W9" s="5" t="inlineStr">
@@ -2130,7 +2126,7 @@
         </is>
       </c>
       <c r="Y9" s="5" t="n">
-        <v>3869319832</v>
+        <v>5824548844</v>
       </c>
       <c r="Z9" s="5" t="inlineStr">
         <is>
@@ -2143,10 +2139,10 @@
         </is>
       </c>
       <c r="AB9" s="5" t="n">
-        <v>245.92</v>
+        <v>404.38</v>
       </c>
       <c r="AC9" s="5" t="n">
-        <v>33.64</v>
+        <v>58.89</v>
       </c>
       <c r="AD9" s="5" t="n">
         <v>0</v>
@@ -2170,7 +2166,7 @@
       </c>
       <c r="AJ9" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível definir o Local de destino!</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK9" s="5" t="inlineStr">
@@ -2180,22 +2176,22 @@
       </c>
       <c r="AL9" s="5" t="inlineStr">
         <is>
-          <t>Cadastro enviado errado no Benner</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM9" s="5" t="inlineStr">
         <is>
-          <t>Cadastro incompleto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN9" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO9" s="5" t="inlineStr">
         <is>
-          <t>Sistêmico</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP9" s="5" t="inlineStr">
@@ -2211,35 +2207,35 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>23082254</v>
+        <v>23336052</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>23833473</v>
+        <v>24064345</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ACC04</t>
+          <t>ACC03</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>45939.90564814815</v>
+        <v>45977.7834375</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>45939.90693287037</v>
+        <v>45979.38715277778</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>IP8YJK</t>
+          <t>BL8JGG</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -2249,7 +2245,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>FRANCISCO FABIO CHAVES OLIVEIRA</t>
+          <t>Felipe Vieira</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -2263,10 +2259,10 @@
         </is>
       </c>
       <c r="M10" s="6" t="n">
-        <v>45939.90486111111</v>
+        <v>45977.78263888889</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>6874856</v>
+        <v>6954301</v>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
@@ -2280,12 +2276,12 @@
       </c>
       <c r="Q10" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão convênio</t>
         </is>
       </c>
       <c r="S10" s="5" t="inlineStr">
@@ -2295,7 +2291,7 @@
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
@@ -2305,7 +2301,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>Glauto da Costa Marques</t>
+          <t>Giulianna Angelica Piason de Brito</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -2319,7 +2315,7 @@
         </is>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>6557544600</v>
+        <v>6776511627</v>
       </c>
       <c r="Z10" s="5" t="inlineStr">
         <is>
@@ -2332,10 +2328,10 @@
         </is>
       </c>
       <c r="AB10" s="5" t="n">
-        <v>245.92</v>
+        <v>404.38</v>
       </c>
       <c r="AC10" s="5" t="n">
-        <v>33.64</v>
+        <v>58.89</v>
       </c>
       <c r="AD10" s="5" t="n">
         <v>0</v>
@@ -2359,7 +2355,7 @@
       </c>
       <c r="AJ10" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível definir o Local de destino!</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK10" s="5" t="inlineStr">
@@ -2369,22 +2365,22 @@
       </c>
       <c r="AL10" s="5" t="inlineStr">
         <is>
-          <t>Cadastro enviado errado no Benner</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM10" s="5" t="inlineStr">
         <is>
-          <t>Cadastro incompleto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN10" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO10" s="5" t="inlineStr">
         <is>
-          <t>Sistêmico</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP10" s="5" t="inlineStr">
@@ -2400,10 +2396,10 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>23079675</v>
+        <v>23336013</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>23831027</v>
+        <v>24064300</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
@@ -2411,24 +2407,24 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>45939.67386574074</v>
+        <v>45977.77516203704</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>45939.67550925926</v>
+        <v>45979.38710648148</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>AQ1HTH</t>
+          <t>GMKD4Q</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -2438,7 +2434,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Carlos Menezes</t>
+          <t>Giullia Delgado</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -2452,10 +2448,10 @@
         </is>
       </c>
       <c r="M11" s="6" t="n">
-        <v>45939.67291666667</v>
+        <v>45977.77430555555</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>6874478</v>
+        <v>6954279</v>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
@@ -2469,12 +2465,12 @@
       </c>
       <c r="Q11" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="R11" s="5" t="inlineStr">
         <is>
-          <t>Cartão de crédito</t>
+          <t>Cartão convênio</t>
         </is>
       </c>
       <c r="S11" s="5" t="inlineStr">
@@ -2484,7 +2480,7 @@
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
@@ -2494,7 +2490,7 @@
       </c>
       <c r="V11" s="5" t="inlineStr">
         <is>
-          <t>Tanise Trevisan</t>
+          <t>Giulianna Angelica Piason de Brito</t>
         </is>
       </c>
       <c r="W11" s="5" t="inlineStr">
@@ -2508,7 +2504,7 @@
         </is>
       </c>
       <c r="Y11" s="5" t="n">
-        <v>5122064463</v>
+        <v>970450104</v>
       </c>
       <c r="Z11" s="5" t="inlineStr">
         <is>
@@ -2521,10 +2517,10 @@
         </is>
       </c>
       <c r="AB11" s="5" t="n">
-        <v>352.42</v>
+        <v>404.38</v>
       </c>
       <c r="AC11" s="5" t="n">
-        <v>60.62</v>
+        <v>58.89</v>
       </c>
       <c r="AD11" s="5" t="n">
         <v>0</v>
@@ -2539,7 +2535,7 @@
         <v>0</v>
       </c>
       <c r="AH11" s="5" t="n">
-        <v>45.24</v>
+        <v>151.32</v>
       </c>
       <c r="AI11" s="5" t="inlineStr">
         <is>
@@ -2548,7 +2544,7 @@
       </c>
       <c r="AJ11" s="5" t="inlineStr">
         <is>
-          <t>Não foi possível definir o Local de destino!</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK11" s="5" t="inlineStr">
@@ -2558,22 +2554,22 @@
       </c>
       <c r="AL11" s="5" t="inlineStr">
         <is>
-          <t>Cadastro enviado errado no Benner</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM11" s="5" t="inlineStr">
         <is>
-          <t>Cadastro incompleto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN11" s="5" t="inlineStr">
         <is>
-          <t>Sistema</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO11" s="5" t="inlineStr">
         <is>
-          <t>Sistêmico</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP11" s="5" t="inlineStr">
@@ -2589,64 +2585,62 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>23078368</v>
+        <v>23336013</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>23829751</v>
+        <v>24064301</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>ACC01</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>45939.56693287037</v>
+        <v>45977.77516203704</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>45939.57008101852</v>
+        <v>45979.38710648148</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>NQ6NXK</t>
+          <t>GMKD4Q</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>ISMARA SILVA</t>
+          <t>Giulianna Brito</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
         <is>
-          <t>Kaique Ferreira Aguiar</t>
+          <t>Zupper</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>Kaique Ferreira Aguiar</t>
+          <t>Zupper</t>
         </is>
       </c>
       <c r="M12" s="6" t="n">
-        <v>45936.56666666667</v>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>45977.77430555555</v>
+      </c>
+      <c r="N12" s="5" t="n">
+        <v>6954279</v>
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
@@ -2675,7 +2669,7 @@
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
@@ -2685,7 +2679,7 @@
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>Zupper Cartao</t>
+          <t>Giulianna Angelica Piason de Brito</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -2699,7 +2693,7 @@
         </is>
       </c>
       <c r="Y12" s="5" t="n">
-        <v>3023829750</v>
+        <v>1961580109</v>
       </c>
       <c r="Z12" s="5" t="inlineStr">
         <is>
@@ -2712,10 +2706,10 @@
         </is>
       </c>
       <c r="AB12" s="5" t="n">
-        <v>521.98</v>
+        <v>404.38</v>
       </c>
       <c r="AC12" s="5" t="n">
-        <v>0</v>
+        <v>58.89</v>
       </c>
       <c r="AD12" s="5" t="n">
         <v>0</v>
@@ -2730,7 +2724,7 @@
         <v>0</v>
       </c>
       <c r="AH12" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="AI12" s="5" t="inlineStr">
         <is>
@@ -2739,7 +2733,7 @@
       </c>
       <c r="AJ12" s="5" t="inlineStr">
         <is>
-          <t>36Faltou informar rateio de centro de custo/projeto abaixo da accounting</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK12" s="5" t="inlineStr">
@@ -2749,22 +2743,22 @@
       </c>
       <c r="AL12" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM12" s="5" t="inlineStr">
         <is>
-          <t>Rateio de centro de custo/projeto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN12" s="5" t="inlineStr">
         <is>
-          <t>Dados Gerenciais</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO12" s="5" t="inlineStr">
         <is>
-          <t>Qualidade dos dados</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP12" s="5" t="inlineStr">
@@ -2780,64 +2774,62 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>23078368</v>
+        <v>23329909</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>23829768</v>
+        <v>24059069</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC03</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>45939.56693287037</v>
+        <v>45976.2847800926</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>45939.57008101852</v>
+        <v>45979.37612268519</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>NQ6NXK</t>
+          <t>CFLRJQ</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>MARCIA COSTA</t>
+          <t>Paulo Vitor Meireles</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>Kaique Ferreira Aguiar</t>
+          <t>Zupper</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>Kaique Ferreira Aguiar</t>
+          <t>Zupper</t>
         </is>
       </c>
       <c r="M13" s="6" t="n">
-        <v>45936.56666666667</v>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>45976.28402777778</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>6951692</v>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
@@ -2866,7 +2858,7 @@
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U13" s="5" t="inlineStr">
@@ -2886,11 +2878,11 @@
       </c>
       <c r="X13" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y13" s="5" t="n">
-        <v>3023829771</v>
+        <v>2259793072</v>
       </c>
       <c r="Z13" s="5" t="inlineStr">
         <is>
@@ -2903,10 +2895,10 @@
         </is>
       </c>
       <c r="AB13" s="5" t="n">
-        <v>521.98</v>
+        <v>577.52</v>
       </c>
       <c r="AC13" s="5" t="n">
-        <v>0</v>
+        <v>55.17</v>
       </c>
       <c r="AD13" s="5" t="n">
         <v>0</v>
@@ -2930,7 +2922,7 @@
       </c>
       <c r="AJ13" s="5" t="inlineStr">
         <is>
-          <t>36Faltou informar rateio de centro de custo/projeto abaixo da accounting</t>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
         </is>
       </c>
       <c r="AK13" s="5" t="inlineStr">
@@ -2940,22 +2932,22 @@
       </c>
       <c r="AL13" s="5" t="inlineStr">
         <is>
-          <t>Falta de informação Gerencial</t>
+          <t>Conciliação de Cartão</t>
         </is>
       </c>
       <c r="AM13" s="5" t="inlineStr">
         <is>
-          <t>Rateio de centro de custo/projeto</t>
+          <t>Financeiro Conciliado</t>
         </is>
       </c>
       <c r="AN13" s="5" t="inlineStr">
         <is>
-          <t>Dados Gerenciais</t>
+          <t>Edição não Permitida</t>
         </is>
       </c>
       <c r="AO13" s="5" t="inlineStr">
         <is>
-          <t>Qualidade dos dados</t>
+          <t>Processo Operacional</t>
         </is>
       </c>
       <c r="AP13" s="5" t="inlineStr">
@@ -2971,64 +2963,62 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>23078572</v>
+        <v>23329909</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>23829974</v>
+        <v>24059070</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ACC</t>
+          <t>ACC04</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>45939.57417824074</v>
+        <v>45976.2847800926</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>45939.57682870371</v>
+        <v>45979.37612268519</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>0 a 02 dias</t>
+          <t>09 a 15 dias</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>LWUQ6K</t>
+          <t>CFLRJQ</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>MANUAL</t>
+          <t>EBOOKING</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>VIVIAN SANCHES</t>
+          <t>Emanuel Ribeiro Franca</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
         <is>
-          <t>Kaique Ferreira Aguiar</t>
+          <t>Zupper</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>Kaique Ferreira Aguiar</t>
+          <t>Zupper</t>
         </is>
       </c>
       <c r="M14" s="6" t="n">
-        <v>45937.57361111111</v>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>45976.28402777778</v>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>6951692</v>
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
@@ -3057,7 +3047,7 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
@@ -3067,7 +3057,7 @@
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>Jorge Artur Leite da Silva Junior</t>
+          <t>Zupper Cartao</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -3077,84 +3067,1974 @@
       </c>
       <c r="X14" s="5" t="inlineStr">
         <is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y14" s="5" t="n">
+        <v>2259793073</v>
+      </c>
+      <c r="Z14" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB14" s="5" t="n">
+        <v>577.52</v>
+      </c>
+      <c r="AC14" s="5" t="n">
+        <v>55.17</v>
+      </c>
+      <c r="AD14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI14" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ14" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK14" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL14" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM14" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN14" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO14" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP14" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ14" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>23329909</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>24059071</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>ACC05</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>45976.2847800926</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>45979.37612268519</v>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>CFLRJQ</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>Ednildo Edgar Goncalves</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>45976.28402777778</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>6951692</v>
+      </c>
+      <c r="O15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R15" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S15" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T15" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U15" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V15" s="5" t="inlineStr">
+        <is>
+          <t>Zupper Cartao</t>
+        </is>
+      </c>
+      <c r="W15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X15" s="5" t="inlineStr">
+        <is>
+          <t>Latam Airlines Brasil</t>
+        </is>
+      </c>
+      <c r="Y15" s="5" t="n">
+        <v>2259793074</v>
+      </c>
+      <c r="Z15" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB15" s="5" t="n">
+        <v>577.52</v>
+      </c>
+      <c r="AC15" s="5" t="n">
+        <v>55.17</v>
+      </c>
+      <c r="AD15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI15" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ15" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK15" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL15" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM15" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN15" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO15" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP15" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ15" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n">
+        <v>23330902</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>24059906</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>ACC01</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>45976.530625</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>45979.37728009259</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>KGVCWI</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Satila Mateus Abrantes</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M16" s="6" t="n">
+        <v>45976.52986111111</v>
+      </c>
+      <c r="N16" s="5" t="n">
+        <v>6952102</v>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U16" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V16" s="5" t="inlineStr">
+        <is>
+          <t>Eduardo Santos da Mata</t>
+        </is>
+      </c>
+      <c r="W16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
           <t>Azul Linhas Aereas</t>
         </is>
       </c>
-      <c r="Y14" s="5" t="n">
-        <v>3023829973</v>
-      </c>
-      <c r="Z14" s="5" t="inlineStr">
+      <c r="Y16" s="5" t="n">
+        <v>9106749780</v>
+      </c>
+      <c r="Z16" s="5" t="inlineStr">
         <is>
           <t>ZUPPER</t>
         </is>
       </c>
-      <c r="AA14" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB14" s="5" t="n">
-        <v>819.8</v>
-      </c>
-      <c r="AC14" s="5" t="n">
-        <v>109.62</v>
-      </c>
-      <c r="AD14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="5" t="n">
-        <v>100</v>
-      </c>
-      <c r="AI14" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AJ14" s="5" t="inlineStr">
-        <is>
-          <t>36Faltou informar rateio de centro de custo/projeto abaixo da accounting</t>
-        </is>
-      </c>
-      <c r="AK14" s="5" t="inlineStr">
+      <c r="AA16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB16" s="5" t="n">
+        <v>1386.67</v>
+      </c>
+      <c r="AC16" s="5" t="n">
+        <v>32.87</v>
+      </c>
+      <c r="AD16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH16" s="5" t="n">
+        <v>169.18</v>
+      </c>
+      <c r="AI16" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ16" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25392354. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK16" s="5" t="inlineStr">
         <is>
           <t>ZUPPER</t>
         </is>
       </c>
-      <c r="AL14" s="5" t="inlineStr">
-        <is>
-          <t>Falta de informação Gerencial</t>
-        </is>
-      </c>
-      <c r="AM14" s="5" t="inlineStr">
-        <is>
-          <t>Rateio de centro de custo/projeto</t>
-        </is>
-      </c>
-      <c r="AN14" s="5" t="inlineStr">
-        <is>
-          <t>Dados Gerenciais</t>
-        </is>
-      </c>
-      <c r="AO14" s="5" t="inlineStr">
-        <is>
-          <t>Qualidade dos dados</t>
-        </is>
-      </c>
-      <c r="AP14" s="5" t="inlineStr">
+      <c r="AL16" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM16" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN16" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO16" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP16" s="5" t="inlineStr">
         <is>
           <t>ZUPPER VIAGENS</t>
         </is>
       </c>
-      <c r="AQ14" s="5" t="inlineStr">
+      <c r="AQ16" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>23336013</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>24064302</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>ACC03</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>45977.77516203704</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>45979.38710648148</v>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>GMKD4Q</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Felipe Vieira</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M17" s="6" t="n">
+        <v>45977.77430555555</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>6954279</v>
+      </c>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S17" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T17" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U17" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V17" s="5" t="inlineStr">
+        <is>
+          <t>Giulianna Angelica Piason de Brito</t>
+        </is>
+      </c>
+      <c r="W17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X17" s="5" t="inlineStr">
+        <is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y17" s="5" t="n">
+        <v>5373137183</v>
+      </c>
+      <c r="Z17" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB17" s="5" t="n">
+        <v>404.38</v>
+      </c>
+      <c r="AC17" s="5" t="n">
+        <v>58.89</v>
+      </c>
+      <c r="AD17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI17" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ17" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK17" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL17" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM17" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN17" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO17" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP17" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ17" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>23336013</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>24064303</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>ACC04</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>45977.77516203704</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>45979.38710648148</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>GMKD4Q</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Rafael Vieira</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M18" s="6" t="n">
+        <v>45977.77430555555</v>
+      </c>
+      <c r="N18" s="5" t="n">
+        <v>6954279</v>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U18" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V18" s="5" t="inlineStr">
+        <is>
+          <t>Giulianna Angelica Piason de Brito</t>
+        </is>
+      </c>
+      <c r="W18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X18" s="5" t="inlineStr">
+        <is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y18" s="5" t="n">
+        <v>2846058807</v>
+      </c>
+      <c r="Z18" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI18" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ18" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK18" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL18" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM18" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN18" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO18" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP18" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ18" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>23336013</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>24064304</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>ACC05</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>45977.77516203704</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>45979.38710648148</v>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>GMKD4Q</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>Luisa Delgado</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>45977.77430555555</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>6954279</v>
+      </c>
+      <c r="O19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P19" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q19" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S19" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T19" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U19" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V19" s="5" t="inlineStr">
+        <is>
+          <t>Giulianna Angelica Piason de Brito</t>
+        </is>
+      </c>
+      <c r="W19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X19" s="5" t="inlineStr">
+        <is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y19" s="5" t="n">
+        <v>2252583666</v>
+      </c>
+      <c r="Z19" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI19" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ19" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK19" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL19" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM19" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN19" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO19" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP19" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ19" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>23336052</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>24064343</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>ACC01</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>45977.7834375</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>45979.38715277778</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>BL8JGG</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Giullia Delgado</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>45977.78263888889</v>
+      </c>
+      <c r="N20" s="5" t="n">
+        <v>6954301</v>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V20" s="5" t="inlineStr">
+        <is>
+          <t>Giulianna Angelica Piason de Brito</t>
+        </is>
+      </c>
+      <c r="W20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X20" s="5" t="inlineStr">
+        <is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="n">
+        <v>3340742969</v>
+      </c>
+      <c r="Z20" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB20" s="5" t="n">
+        <v>404.38</v>
+      </c>
+      <c r="AC20" s="5" t="n">
+        <v>58.89</v>
+      </c>
+      <c r="AD20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH20" s="5" t="n">
+        <v>151.32</v>
+      </c>
+      <c r="AI20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ20" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK20" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL20" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM20" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN20" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO20" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP20" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ20" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>23336392</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>24064696</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>ACC01</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>45977.85212962963</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>45979.38746527778</v>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>MJ7MKP</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>Jose Figueiredo</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>45977.85138888889</v>
+      </c>
+      <c r="N21" s="5" t="n">
+        <v>6954464</v>
+      </c>
+      <c r="O21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P21" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q21" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S21" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T21" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U21" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V21" s="5" t="inlineStr">
+        <is>
+          <t>Jose Antonio de Figueiredo</t>
+        </is>
+      </c>
+      <c r="W21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X21" s="5" t="inlineStr">
+        <is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y21" s="5" t="n">
+        <v>9825033326</v>
+      </c>
+      <c r="Z21" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB21" s="5" t="n">
+        <v>1662.64</v>
+      </c>
+      <c r="AC21" s="5" t="n">
+        <v>39.58</v>
+      </c>
+      <c r="AD21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH21" s="5" t="n">
+        <v>405.68</v>
+      </c>
+      <c r="AI21" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ21" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395732. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK21" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL21" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM21" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN21" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO21" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP21" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ21" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>23336392</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>24064697</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>ACC02</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>45977.85212962963</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>45979.38746527778</v>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>MJ7MKP</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Kelmey Santos</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M22" s="6" t="n">
+        <v>45977.85138888889</v>
+      </c>
+      <c r="N22" s="5" t="n">
+        <v>6954464</v>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S22" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V22" s="5" t="inlineStr">
+        <is>
+          <t>Jose Antonio de Figueiredo</t>
+        </is>
+      </c>
+      <c r="W22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X22" s="5" t="inlineStr">
+        <is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y22" s="5" t="n">
+        <v>1720811985</v>
+      </c>
+      <c r="Z22" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB22" s="5" t="n">
+        <v>1662.64</v>
+      </c>
+      <c r="AC22" s="5" t="n">
+        <v>39.58</v>
+      </c>
+      <c r="AD22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI22" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ22" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395732. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK22" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL22" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM22" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN22" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO22" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP22" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ22" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>23336052</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>24064346</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>ACC04</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>45977.7834375</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>45979.38715277778</v>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>BL8JGG</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>Rafael Vieira</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>45977.78263888889</v>
+      </c>
+      <c r="N23" s="5" t="n">
+        <v>6954301</v>
+      </c>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P23" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q23" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S23" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T23" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U23" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V23" s="5" t="inlineStr">
+        <is>
+          <t>Giulianna Angelica Piason de Brito</t>
+        </is>
+      </c>
+      <c r="W23" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X23" s="5" t="inlineStr">
+        <is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y23" s="5" t="n">
+        <v>4961395002</v>
+      </c>
+      <c r="Z23" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA23" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI23" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ23" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK23" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL23" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM23" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN23" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO23" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP23" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ23" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>23336052</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>24064347</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>ACC05</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>45977.7834375</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>45979.38715277778</v>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>06 a 08 dias</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>09 a 15 dias</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>BL8JGG</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>Luisa Delgado</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>45977.78263888889</v>
+      </c>
+      <c r="N24" s="5" t="n">
+        <v>6954301</v>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S24" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T24" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="U24" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V24" s="5" t="inlineStr">
+        <is>
+          <t>Giulianna Angelica Piason de Brito</t>
+        </is>
+      </c>
+      <c r="W24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X24" s="5" t="inlineStr">
+        <is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y24" s="5" t="n">
+        <v>2175324568</v>
+      </c>
+      <c r="Z24" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI24" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ24" s="5" t="inlineStr">
+        <is>
+          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+        </is>
+      </c>
+      <c r="AK24" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL24" s="5" t="inlineStr">
+        <is>
+          <t>Conciliação de Cartão</t>
+        </is>
+      </c>
+      <c r="AM24" s="5" t="inlineStr">
+        <is>
+          <t>Financeiro Conciliado</t>
+        </is>
+      </c>
+      <c r="AN24" s="5" t="inlineStr">
+        <is>
+          <t>Edição não Permitida</t>
+        </is>
+      </c>
+      <c r="AO24" s="5" t="inlineStr">
+        <is>
+          <t>Processo Operacional</t>
+        </is>
+      </c>
+      <c r="AP24" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ24" s="5" t="inlineStr">
         <is>
           <t>Operações - ZUPPER</t>
         </is>

</xml_diff>

<commit_message>
Fix error processing, adjust email body, add reports
Fix Python logic and email content: remove stray comment in 2-processamento_erros.py so the 'Rateio de centro de custo/projeto' condition is applied correctly, and remove corpo_email_2 from the HTML body for KONTIK/GRUPO KONTIK in 4-envio_relatorios.py to simplify the sent emails. Update integration artifacts: multiple Excel report files were updated and numerous PDF reports were added under Integration-Quality/PDFs. These changes ensure correct error categorization and refresh generated report assets.
</commit_message>
<xml_diff>
--- a/Integration-Quality/EMPRESAS/Relatorio - ZUPPER VIAGENS.xlsx
+++ b/Integration-Quality/EMPRESAS/Relatorio - ZUPPER VIAGENS.xlsx
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ24"/>
+  <dimension ref="A1:AQ25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -695,10 +695,10 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>23378056</v>
+        <v>24508519</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>24101850</v>
+        <v>25322829</v>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
@@ -706,10 +706,10 @@
         </is>
       </c>
       <c r="D2" s="6" t="n">
-        <v>45985.3716087963</v>
+        <v>46139.82451388889</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>45985.37324074074</v>
+        <v>46139.82570601852</v>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
@@ -723,7 +723,7 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>UICKQU</t>
+          <t>UMBAHM</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>MARIA CLAUDIA PINHEIRO</t>
+          <t>Antonio Goncalves</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -747,10 +747,10 @@
         </is>
       </c>
       <c r="M2" s="6" t="n">
-        <v>45985.37083333333</v>
+        <v>46139.82361111111</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>6976871</v>
+        <v>7370397</v>
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
@@ -784,12 +784,12 @@
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Grupo Zupper</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>Maria Claudia Costa Paunovic</t>
+          <t>Antonio Silva Goncalves</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -803,7 +803,7 @@
         </is>
       </c>
       <c r="Y2" s="5" t="n">
-        <v>2150095851</v>
+        <v>2302659398</v>
       </c>
       <c r="Z2" s="5" t="inlineStr">
         <is>
@@ -816,10 +816,10 @@
         </is>
       </c>
       <c r="AB2" s="5" t="n">
-        <v>448.73</v>
+        <v>486.01</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>56.88</v>
+        <v>34.11</v>
       </c>
       <c r="AD2" s="5" t="n">
         <v>0</v>
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>44.87</v>
+        <v>44.74</v>
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
@@ -843,7 +843,7 @@
       </c>
       <c r="AJ2" s="5" t="inlineStr">
         <is>
-          <t>Necessário cadastrar um contrato para o cliente ""</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK2" s="5" t="inlineStr">
@@ -853,22 +853,22 @@
       </c>
       <c r="AL2" s="5" t="inlineStr">
         <is>
-          <t>Contrato de fornecedor</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM2" s="5" t="inlineStr">
         <is>
-          <t>Análise Cadastro</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN2" s="5" t="inlineStr">
         <is>
-          <t>Dados do Fornecedor</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO2" s="5" t="inlineStr">
         <is>
-          <t>Qualidade dos dados</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP2" s="5" t="inlineStr">
@@ -884,10 +884,10 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
-        <v>23379736</v>
+        <v>24509411</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>24103425</v>
+        <v>25323900</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -895,10 +895,10 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>45985.63831018518</v>
+        <v>46139.90917824074</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>45985.63976851852</v>
+        <v>46139.91130787037</v>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
@@ -912,7 +912,7 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>NFJUSP</t>
+          <t>QZSWFM</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Julio Cesar Silva Junior</t>
+          <t>MARIA ILZA MARTINS</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -936,10 +936,10 @@
         </is>
       </c>
       <c r="M3" s="6" t="n">
-        <v>45985.6375</v>
+        <v>46139.90833333333</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>6977313</v>
+        <v>7370847</v>
       </c>
       <c r="O3" s="5" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
       </c>
       <c r="V3" s="5" t="inlineStr">
         <is>
-          <t>Priscila Cortez Braga Silva</t>
+          <t>Monica Welfer</t>
         </is>
       </c>
       <c r="W3" s="5" t="inlineStr">
@@ -988,11 +988,11 @@
       </c>
       <c r="X3" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y3" s="5" t="n">
-        <v>2261090024</v>
+        <v>2302668528</v>
       </c>
       <c r="Z3" s="5" t="inlineStr">
         <is>
@@ -1005,10 +1005,10 @@
         </is>
       </c>
       <c r="AB3" s="5" t="n">
-        <v>769.52</v>
+        <v>695.11</v>
       </c>
       <c r="AC3" s="5" t="n">
-        <v>56.78</v>
+        <v>38.39</v>
       </c>
       <c r="AD3" s="5" t="n">
         <v>0</v>
@@ -1023,7 +1023,7 @@
         <v>0</v>
       </c>
       <c r="AH3" s="5" t="n">
-        <v>230.86</v>
+        <v>63.56</v>
       </c>
       <c r="AI3" s="5" t="inlineStr">
         <is>
@@ -1073,10 +1073,10 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>23329909</v>
+        <v>24477696</v>
       </c>
       <c r="B4" s="5" t="n">
-        <v>24059067</v>
+        <v>25285769</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -1084,10 +1084,10 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>45976.2847800926</v>
+        <v>46133.19391203704</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>45979.37612268519</v>
+        <v>46135.82152777778</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -1096,12 +1096,12 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>CFLRJQ</t>
+          <t>NEIJWU</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>Rosenir Silva Braga</t>
+          <t>Mercia Alapenha</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1125,10 +1125,10 @@
         </is>
       </c>
       <c r="M4" s="6" t="n">
-        <v>45976.28402777778</v>
+        <v>46133.19305555556</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>6951692</v>
+        <v>7353196</v>
       </c>
       <c r="O4" s="5" t="inlineStr">
         <is>
@@ -1142,12 +1142,12 @@
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>Cartão convênio</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S4" s="5" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>Zupper Cartao</t>
+          <t>Diego B Silva</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1177,11 +1177,11 @@
       </c>
       <c r="X4" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>2259793070</v>
+        <v>2302258124</v>
       </c>
       <c r="Z4" s="5" t="inlineStr">
         <is>
@@ -1194,10 +1194,10 @@
         </is>
       </c>
       <c r="AB4" s="5" t="n">
-        <v>577.52</v>
+        <v>703.21</v>
       </c>
       <c r="AC4" s="5" t="n">
-        <v>55.17</v>
+        <v>52.72</v>
       </c>
       <c r="AD4" s="5" t="n">
         <v>0</v>
@@ -1212,7 +1212,7 @@
         <v>0</v>
       </c>
       <c r="AH4" s="5" t="n">
-        <v>490.9</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="AI4" s="5" t="inlineStr">
         <is>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="AJ4" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t xml:space="preserve">Erro excluindo PNR: Não é possivel excluir a accounting de código: 26321625. A mesma está ligada a conciliação de cartão "ANTECIPAÇÃO REDE </t>
         </is>
       </c>
       <c r="AK4" s="5" t="inlineStr">
@@ -1262,21 +1262,21 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>23329909</v>
+        <v>24484498</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>24059068</v>
+        <v>25294456</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>45976.2847800926</v>
+        <v>46134.7300925926</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>45979.37612268519</v>
+        <v>46135.87565972222</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -1285,12 +1285,12 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>06 a 08 dias</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>CFLRJQ</t>
+          <t>AQWQZC</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>Girleno Menezes Barbosa</t>
+          <t>KELVIN DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
@@ -1314,10 +1314,10 @@
         </is>
       </c>
       <c r="M5" s="6" t="n">
-        <v>45976.28402777778</v>
+        <v>46134.72916666666</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>6951692</v>
+        <v>7357558</v>
       </c>
       <c r="O5" s="5" t="inlineStr">
         <is>
@@ -1331,12 +1331,12 @@
       </c>
       <c r="Q5" s="5" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>Cartão convênio</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S5" s="5" t="inlineStr">
@@ -1366,11 +1366,11 @@
       </c>
       <c r="X5" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>2259793071</v>
+        <v>2302351359</v>
       </c>
       <c r="Z5" s="5" t="inlineStr">
         <is>
@@ -1383,10 +1383,10 @@
         </is>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>577.52</v>
+        <v>1566.42</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>55.17</v>
+        <v>92.33</v>
       </c>
       <c r="AD5" s="5" t="n">
         <v>0</v>
@@ -1401,7 +1401,7 @@
         <v>0</v>
       </c>
       <c r="AH5" s="5" t="n">
-        <v>0</v>
+        <v>214.66</v>
       </c>
       <c r="AI5" s="5" t="inlineStr">
         <is>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="AJ5" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t xml:space="preserve">Erro excluindo PNR: Não é possivel excluir a accounting de código: 26330553. A mesma está ligada a conciliação de cartão "ANTECIPAÇÃO REDE </t>
         </is>
       </c>
       <c r="AK5" s="5" t="inlineStr">
@@ -1451,10 +1451,10 @@
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
-        <v>23332722</v>
+        <v>24505405</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>24061614</v>
+        <v>25319277</v>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
@@ -1462,24 +1462,24 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>45976.91744212963</v>
+        <v>46139.5515162037</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>45979.37971064815</v>
+        <v>46139.55336805555</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>RLZEGZ</t>
+          <t>QMITMH</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>ADEMIR VALERIO</t>
+          <t>Anderson Mello</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1503,10 +1503,10 @@
         </is>
       </c>
       <c r="M6" s="6" t="n">
-        <v>45976.91666666666</v>
+        <v>46139.55069444444</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>6952979</v>
+        <v>7369316</v>
       </c>
       <c r="O6" s="5" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>Fabiana Sambini</t>
+          <t>Anderson Marcelo Mello</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1555,11 +1555,11 @@
       </c>
       <c r="X6" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y6" s="5" t="n">
-        <v>3895134748</v>
+        <v>2302630905</v>
       </c>
       <c r="Z6" s="5" t="inlineStr">
         <is>
@@ -1572,10 +1572,10 @@
         </is>
       </c>
       <c r="AB6" s="5" t="n">
-        <v>1682.08</v>
+        <v>698.21</v>
       </c>
       <c r="AC6" s="5" t="n">
-        <v>92.53</v>
+        <v>59.46</v>
       </c>
       <c r="AD6" s="5" t="n">
         <v>0</v>
@@ -1590,7 +1590,7 @@
         <v>0</v>
       </c>
       <c r="AH6" s="5" t="n">
-        <v>0</v>
+        <v>49.87</v>
       </c>
       <c r="AI6" s="5" t="inlineStr">
         <is>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="AJ6" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25393682. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK6" s="5" t="inlineStr">
@@ -1609,22 +1609,22 @@
       </c>
       <c r="AL6" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM6" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN6" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO6" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP6" s="5" t="inlineStr">
@@ -1640,10 +1640,10 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>23333521</v>
+        <v>24506539</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>24062221</v>
+        <v>25320579</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -1651,24 +1651,24 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>45977.14121527778</v>
+        <v>46139.64179398148</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>45979.38116898148</v>
+        <v>46139.64315972223</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>WFYUWK</t>
+          <t>WKXOOR</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -1678,7 +1678,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Victoria Cruz</t>
+          <t>ELIANE LIMA</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
@@ -1692,10 +1692,10 @@
         </is>
       </c>
       <c r="M7" s="6" t="n">
-        <v>45977.14027777778</v>
+        <v>46139.64097222222</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>6953294</v>
+        <v>7369655</v>
       </c>
       <c r="O7" s="5" t="inlineStr">
         <is>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="T7" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U7" s="5" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="V7" s="5" t="inlineStr">
         <is>
-          <t>Zupper Cartao</t>
+          <t>Eliane Guedes de Moura Lima</t>
         </is>
       </c>
       <c r="W7" s="5" t="inlineStr">
@@ -1744,11 +1744,11 @@
       </c>
       <c r="X7" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>2259897267</v>
+        <v>2302639428</v>
       </c>
       <c r="Z7" s="5" t="inlineStr">
         <is>
@@ -1761,10 +1761,10 @@
         </is>
       </c>
       <c r="AB7" s="5" t="n">
-        <v>1052.72</v>
+        <v>498.07</v>
       </c>
       <c r="AC7" s="5" t="n">
-        <v>56.78</v>
+        <v>54.09</v>
       </c>
       <c r="AD7" s="5" t="n">
         <v>0</v>
@@ -1779,7 +1779,7 @@
         <v>0</v>
       </c>
       <c r="AH7" s="5" t="n">
-        <v>357.92</v>
+        <v>212.96</v>
       </c>
       <c r="AI7" s="5" t="inlineStr">
         <is>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="AJ7" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25394052. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK7" s="5" t="inlineStr">
@@ -1798,22 +1798,22 @@
       </c>
       <c r="AL7" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM7" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN7" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO7" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP7" s="5" t="inlineStr">
@@ -1829,10 +1829,10 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>23333521</v>
+        <v>24506539</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>24062222</v>
+        <v>25320581</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
@@ -1840,24 +1840,24 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>45977.14121527778</v>
+        <v>46139.64179398148</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>45979.38116898148</v>
+        <v>46139.64315972223</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>WFYUWK</t>
+          <t>WKXOOR</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Benicio Oliveira</t>
+          <t>SEBASTIAO PESSOA</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1881,10 +1881,10 @@
         </is>
       </c>
       <c r="M8" s="6" t="n">
-        <v>45977.14027777778</v>
+        <v>46139.64097222222</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>6953294</v>
+        <v>7369655</v>
       </c>
       <c r="O8" s="5" t="inlineStr">
         <is>
@@ -1913,7 +1913,7 @@
       </c>
       <c r="T8" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U8" s="5" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>Zupper Cartao</t>
+          <t>Eliane Guedes de Moura Lima</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="X8" s="5" t="inlineStr">
         <is>
-          <t>Latam Airlines Brasil</t>
+          <t>Gol Linhas Aereas</t>
         </is>
       </c>
       <c r="Y8" s="5" t="n">
-        <v>2259897268</v>
+        <v>2302639429</v>
       </c>
       <c r="Z8" s="5" t="inlineStr">
         <is>
@@ -1950,10 +1950,10 @@
         </is>
       </c>
       <c r="AB8" s="5" t="n">
-        <v>1052.72</v>
+        <v>498.07</v>
       </c>
       <c r="AC8" s="5" t="n">
-        <v>56.78</v>
+        <v>54.09</v>
       </c>
       <c r="AD8" s="5" t="n">
         <v>0</v>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="AJ8" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25394052. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK8" s="5" t="inlineStr">
@@ -1987,22 +1987,22 @@
       </c>
       <c r="AL8" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM8" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN8" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO8" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP8" s="5" t="inlineStr">
@@ -2018,35 +2018,35 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>23336052</v>
+        <v>24506545</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>24064344</v>
+        <v>25320585</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>ACC02</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>45977.7834375</v>
+        <v>46139.64251157407</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>45979.38715277778</v>
+        <v>46139.64461805556</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>BL8JGG</t>
+          <t>WMNZUC</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -2056,7 +2056,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Delgado</t>
+          <t>ELIANE LIMA</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
@@ -2070,10 +2070,10 @@
         </is>
       </c>
       <c r="M9" s="6" t="n">
-        <v>45977.78263888889</v>
+        <v>46139.64166666667</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>6954301</v>
+        <v>7369656</v>
       </c>
       <c r="O9" s="5" t="inlineStr">
         <is>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U9" s="5" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="V9" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Eliane Guedes de Moura Lima</t>
         </is>
       </c>
       <c r="W9" s="5" t="inlineStr">
@@ -2122,11 +2122,11 @@
       </c>
       <c r="X9" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y9" s="5" t="n">
-        <v>5824548844</v>
+        <v>2284330870</v>
       </c>
       <c r="Z9" s="5" t="inlineStr">
         <is>
@@ -2139,10 +2139,10 @@
         </is>
       </c>
       <c r="AB9" s="5" t="n">
-        <v>404.38</v>
+        <v>433.12</v>
       </c>
       <c r="AC9" s="5" t="n">
-        <v>58.89</v>
+        <v>49.18</v>
       </c>
       <c r="AD9" s="5" t="n">
         <v>0</v>
@@ -2157,7 +2157,7 @@
         <v>0</v>
       </c>
       <c r="AH9" s="5" t="n">
-        <v>0</v>
+        <v>234.51</v>
       </c>
       <c r="AI9" s="5" t="inlineStr">
         <is>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="AJ9" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK9" s="5" t="inlineStr">
@@ -2176,22 +2176,22 @@
       </c>
       <c r="AL9" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM9" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN9" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO9" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP9" s="5" t="inlineStr">
@@ -2207,35 +2207,35 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>23336052</v>
+        <v>24506545</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>24064345</v>
+        <v>25320587</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>ACC03</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>45977.7834375</v>
+        <v>46139.64251157407</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>45979.38715277778</v>
+        <v>46139.64461805556</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>BL8JGG</t>
+          <t>WMNZUC</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Felipe Vieira</t>
+          <t>SEBASTIAO PESSOA</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -2259,10 +2259,10 @@
         </is>
       </c>
       <c r="M10" s="6" t="n">
-        <v>45977.78263888889</v>
+        <v>46139.64166666667</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>6954301</v>
+        <v>7369656</v>
       </c>
       <c r="O10" s="5" t="inlineStr">
         <is>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Eliane Guedes de Moura Lima</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -2311,11 +2311,11 @@
       </c>
       <c r="X10" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>6776511627</v>
+        <v>2284330871</v>
       </c>
       <c r="Z10" s="5" t="inlineStr">
         <is>
@@ -2328,10 +2328,10 @@
         </is>
       </c>
       <c r="AB10" s="5" t="n">
-        <v>404.38</v>
+        <v>433.12</v>
       </c>
       <c r="AC10" s="5" t="n">
-        <v>58.89</v>
+        <v>49.18</v>
       </c>
       <c r="AD10" s="5" t="n">
         <v>0</v>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="AJ10" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK10" s="5" t="inlineStr">
@@ -2365,22 +2365,22 @@
       </c>
       <c r="AL10" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM10" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN10" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO10" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP10" s="5" t="inlineStr">
@@ -2396,10 +2396,10 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>23336013</v>
+        <v>24509165</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>24064300</v>
+        <v>25323525</v>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
@@ -2407,24 +2407,24 @@
         </is>
       </c>
       <c r="D11" s="6" t="n">
-        <v>45977.77516203704</v>
+        <v>46139.86328703703</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>45979.38710648148</v>
+        <v>46139.86543981481</v>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>GMKD4Q</t>
+          <t>DEYQMW</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
@@ -2434,7 +2434,7 @@
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Giullia Delgado</t>
+          <t>Roberta Oliveira Santos</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
@@ -2448,10 +2448,10 @@
         </is>
       </c>
       <c r="M11" s="6" t="n">
-        <v>45977.77430555555</v>
+        <v>46139.8625</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>6954279</v>
+        <v>7370549</v>
       </c>
       <c r="O11" s="5" t="inlineStr">
         <is>
@@ -2465,12 +2465,12 @@
       </c>
       <c r="Q11" s="5" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="R11" s="5" t="inlineStr">
         <is>
-          <t>Cartão convênio</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S11" s="5" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="V11" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Rosalia Maria Oliveira Santos da Silva</t>
         </is>
       </c>
       <c r="W11" s="5" t="inlineStr">
@@ -2500,11 +2500,11 @@
       </c>
       <c r="X11" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y11" s="5" t="n">
-        <v>970450104</v>
+        <v>2284391888</v>
       </c>
       <c r="Z11" s="5" t="inlineStr">
         <is>
@@ -2517,10 +2517,10 @@
         </is>
       </c>
       <c r="AB11" s="5" t="n">
-        <v>404.38</v>
+        <v>528.8</v>
       </c>
       <c r="AC11" s="5" t="n">
-        <v>58.89</v>
+        <v>86.83</v>
       </c>
       <c r="AD11" s="5" t="n">
         <v>0</v>
@@ -2535,7 +2535,7 @@
         <v>0</v>
       </c>
       <c r="AH11" s="5" t="n">
-        <v>151.32</v>
+        <v>503.97</v>
       </c>
       <c r="AI11" s="5" t="inlineStr">
         <is>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="AJ11" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK11" s="5" t="inlineStr">
@@ -2554,22 +2554,22 @@
       </c>
       <c r="AL11" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM11" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN11" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO11" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP11" s="5" t="inlineStr">
@@ -2585,10 +2585,10 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>23336013</v>
+        <v>24509165</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>24064301</v>
+        <v>25323526</v>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
@@ -2596,24 +2596,24 @@
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>45977.77516203704</v>
+        <v>46139.86328703703</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>45979.38710648148</v>
+        <v>46139.86543981481</v>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>GMKD4Q</t>
+          <t>DEYQMW</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
@@ -2623,7 +2623,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Brito</t>
+          <t>Rosalia Maria Silva</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -2637,10 +2637,10 @@
         </is>
       </c>
       <c r="M12" s="6" t="n">
-        <v>45977.77430555555</v>
+        <v>46139.8625</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>6954279</v>
+        <v>7370549</v>
       </c>
       <c r="O12" s="5" t="inlineStr">
         <is>
@@ -2654,12 +2654,12 @@
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr">
         <is>
-          <t>Cartão convênio</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S12" s="5" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Rosalia Maria Oliveira Santos da Silva</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -2689,11 +2689,11 @@
       </c>
       <c r="X12" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y12" s="5" t="n">
-        <v>1961580109</v>
+        <v>2284391889</v>
       </c>
       <c r="Z12" s="5" t="inlineStr">
         <is>
@@ -2706,10 +2706,10 @@
         </is>
       </c>
       <c r="AB12" s="5" t="n">
-        <v>404.38</v>
+        <v>528.8</v>
       </c>
       <c r="AC12" s="5" t="n">
-        <v>58.89</v>
+        <v>86.83</v>
       </c>
       <c r="AD12" s="5" t="n">
         <v>0</v>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="AJ12" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK12" s="5" t="inlineStr">
@@ -2743,22 +2743,22 @@
       </c>
       <c r="AL12" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM12" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN12" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO12" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP12" s="5" t="inlineStr">
@@ -2774,10 +2774,10 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>23329909</v>
+        <v>24509165</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>24059069</v>
+        <v>25323527</v>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
@@ -2785,24 +2785,24 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>45976.2847800926</v>
+        <v>46139.86328703703</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>45979.37612268519</v>
+        <v>46139.86543981481</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>CFLRJQ</t>
+          <t>DEYQMW</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Paulo Vitor Meireles</t>
+          <t>Jose Carlos da Silva</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -2826,10 +2826,10 @@
         </is>
       </c>
       <c r="M13" s="6" t="n">
-        <v>45976.28402777778</v>
+        <v>46139.8625</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>6951692</v>
+        <v>7370549</v>
       </c>
       <c r="O13" s="5" t="inlineStr">
         <is>
@@ -2843,12 +2843,12 @@
       </c>
       <c r="Q13" s="5" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="R13" s="5" t="inlineStr">
         <is>
-          <t>Cartão convênio</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S13" s="5" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="T13" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U13" s="5" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="V13" s="5" t="inlineStr">
         <is>
-          <t>Zupper Cartao</t>
+          <t>Rosalia Maria Oliveira Santos da Silva</t>
         </is>
       </c>
       <c r="W13" s="5" t="inlineStr">
@@ -2882,7 +2882,7 @@
         </is>
       </c>
       <c r="Y13" s="5" t="n">
-        <v>2259793072</v>
+        <v>2284391890</v>
       </c>
       <c r="Z13" s="5" t="inlineStr">
         <is>
@@ -2895,10 +2895,10 @@
         </is>
       </c>
       <c r="AB13" s="5" t="n">
-        <v>577.52</v>
+        <v>528.8</v>
       </c>
       <c r="AC13" s="5" t="n">
-        <v>55.17</v>
+        <v>86.83</v>
       </c>
       <c r="AD13" s="5" t="n">
         <v>0</v>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="AJ13" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK13" s="5" t="inlineStr">
@@ -2932,22 +2932,22 @@
       </c>
       <c r="AL13" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM13" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN13" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO13" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP13" s="5" t="inlineStr">
@@ -2963,35 +2963,35 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>23329909</v>
+        <v>24509930</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>24059070</v>
+        <v>25324662</v>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>ACC04</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>45976.2847800926</v>
+        <v>46140.05016203703</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>45979.37612268519</v>
+        <v>46140.05239583334</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>CFLRJQ</t>
+          <t>QSKVAA</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Emanuel Ribeiro Franca</t>
+          <t>Carlos Oliveira</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -3015,10 +3015,10 @@
         </is>
       </c>
       <c r="M14" s="6" t="n">
-        <v>45976.28402777778</v>
+        <v>46140.04930555556</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>6951692</v>
+        <v>7371500</v>
       </c>
       <c r="O14" s="5" t="inlineStr">
         <is>
@@ -3032,12 +3032,12 @@
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>Invoice</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>Cartão convênio</t>
+          <t>Cartão de crédito</t>
         </is>
       </c>
       <c r="S14" s="5" t="inlineStr">
@@ -3047,7 +3047,7 @@
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>Zupper Cartao</t>
+          <t>Carlos Rogerio de Oliveira</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -3071,7 +3071,7 @@
         </is>
       </c>
       <c r="Y14" s="5" t="n">
-        <v>2259793073</v>
+        <v>2284428457</v>
       </c>
       <c r="Z14" s="5" t="inlineStr">
         <is>
@@ -3084,10 +3084,10 @@
         </is>
       </c>
       <c r="AB14" s="5" t="n">
-        <v>577.52</v>
+        <v>597.28</v>
       </c>
       <c r="AC14" s="5" t="n">
-        <v>55.17</v>
+        <v>48.26</v>
       </c>
       <c r="AD14" s="5" t="n">
         <v>0</v>
@@ -3102,7 +3102,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="5" t="n">
-        <v>0</v>
+        <v>189.62</v>
       </c>
       <c r="AI14" s="5" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="AJ14" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK14" s="5" t="inlineStr">
@@ -3121,22 +3121,22 @@
       </c>
       <c r="AL14" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM14" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN14" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO14" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP14" s="5" t="inlineStr">
@@ -3152,35 +3152,35 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>23329909</v>
+        <v>24506345</v>
       </c>
       <c r="B15" s="5" t="n">
-        <v>24059071</v>
+        <v>25320346</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>ACC05</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>45976.2847800926</v>
+        <v>46139.61607638889</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>45979.37612268519</v>
+        <v>46139.61728009259</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>CFLRJQ</t>
+          <t>UBDNZP</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>Ednildo Edgar Goncalves</t>
+          <t>Jordana jorgelino</t>
         </is>
       </c>
       <c r="K15" s="5" t="inlineStr">
@@ -3204,10 +3204,10 @@
         </is>
       </c>
       <c r="M15" s="6" t="n">
-        <v>45976.28402777778</v>
+        <v>46139.61527777778</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>6951692</v>
+        <v>7369565</v>
       </c>
       <c r="O15" s="5" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="V15" s="5" t="inlineStr">
         <is>
-          <t>Zupper Cartao</t>
+          <t>Jordana Rocha Jorgelino</t>
         </is>
       </c>
       <c r="W15" s="5" t="inlineStr">
@@ -3260,7 +3260,7 @@
         </is>
       </c>
       <c r="Y15" s="5" t="n">
-        <v>2259793074</v>
+        <v>2284323768</v>
       </c>
       <c r="Z15" s="5" t="inlineStr">
         <is>
@@ -3273,10 +3273,10 @@
         </is>
       </c>
       <c r="AB15" s="5" t="n">
-        <v>577.52</v>
+        <v>660.36</v>
       </c>
       <c r="AC15" s="5" t="n">
-        <v>55.17</v>
+        <v>31.73</v>
       </c>
       <c r="AD15" s="5" t="n">
         <v>0</v>
@@ -3291,7 +3291,7 @@
         <v>0</v>
       </c>
       <c r="AH15" s="5" t="n">
-        <v>0</v>
+        <v>209.54</v>
       </c>
       <c r="AI15" s="5" t="inlineStr">
         <is>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="AJ15" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25391809. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK15" s="5" t="inlineStr">
@@ -3310,22 +3310,22 @@
       </c>
       <c r="AL15" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM15" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN15" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO15" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP15" s="5" t="inlineStr">
@@ -3341,10 +3341,10 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="n">
-        <v>23330902</v>
+        <v>24506633</v>
       </c>
       <c r="B16" s="5" t="n">
-        <v>24059906</v>
+        <v>25320681</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
@@ -3352,24 +3352,24 @@
         </is>
       </c>
       <c r="D16" s="6" t="n">
-        <v>45976.530625</v>
+        <v>46139.65355324074</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>45979.37728009259</v>
+        <v>46139.65498842593</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>KGVCWI</t>
+          <t>WGXDQS</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Satila Mateus Abrantes</t>
+          <t>Cleizer Bessa</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -3393,10 +3393,10 @@
         </is>
       </c>
       <c r="M16" s="6" t="n">
-        <v>45976.52986111111</v>
+        <v>46139.65277777778</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>6952102</v>
+        <v>7369681</v>
       </c>
       <c r="O16" s="5" t="inlineStr">
         <is>
@@ -3425,7 +3425,7 @@
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>Eduardo Santos da Mata</t>
+          <t>Cleizer</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -3445,11 +3445,11 @@
       </c>
       <c r="X16" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y16" s="5" t="n">
-        <v>9106749780</v>
+        <v>2284334233</v>
       </c>
       <c r="Z16" s="5" t="inlineStr">
         <is>
@@ -3462,10 +3462,10 @@
         </is>
       </c>
       <c r="AB16" s="5" t="n">
-        <v>1386.67</v>
+        <v>554.72</v>
       </c>
       <c r="AC16" s="5" t="n">
-        <v>32.87</v>
+        <v>34.11</v>
       </c>
       <c r="AD16" s="5" t="n">
         <v>0</v>
@@ -3480,7 +3480,7 @@
         <v>0</v>
       </c>
       <c r="AH16" s="5" t="n">
-        <v>169.18</v>
+        <v>135.14</v>
       </c>
       <c r="AI16" s="5" t="inlineStr">
         <is>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="AJ16" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25392354. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK16" s="5" t="inlineStr">
@@ -3499,22 +3499,22 @@
       </c>
       <c r="AL16" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM16" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN16" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO16" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP16" s="5" t="inlineStr">
@@ -3530,35 +3530,35 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>23336013</v>
+        <v>24506633</v>
       </c>
       <c r="B17" s="5" t="n">
-        <v>24064302</v>
+        <v>25320682</v>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>ACC03</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>45977.77516203704</v>
+        <v>46139.65355324074</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>45979.38710648148</v>
+        <v>46139.65498842593</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>GMKD4Q</t>
+          <t>WGXDQS</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
@@ -3568,7 +3568,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Felipe Vieira</t>
+          <t>Carlos Henrique Santos</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -3582,10 +3582,10 @@
         </is>
       </c>
       <c r="M17" s="6" t="n">
-        <v>45977.77430555555</v>
+        <v>46139.65277777778</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>6954279</v>
+        <v>7369681</v>
       </c>
       <c r="O17" s="5" t="inlineStr">
         <is>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="T17" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U17" s="5" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="V17" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Cleizer</t>
         </is>
       </c>
       <c r="W17" s="5" t="inlineStr">
@@ -3634,11 +3634,11 @@
       </c>
       <c r="X17" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y17" s="5" t="n">
-        <v>5373137183</v>
+        <v>2284334234</v>
       </c>
       <c r="Z17" s="5" t="inlineStr">
         <is>
@@ -3651,10 +3651,10 @@
         </is>
       </c>
       <c r="AB17" s="5" t="n">
-        <v>404.38</v>
+        <v>554.72</v>
       </c>
       <c r="AC17" s="5" t="n">
-        <v>58.89</v>
+        <v>34.11</v>
       </c>
       <c r="AD17" s="5" t="n">
         <v>0</v>
@@ -3678,7 +3678,7 @@
       </c>
       <c r="AJ17" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK17" s="5" t="inlineStr">
@@ -3688,22 +3688,22 @@
       </c>
       <c r="AL17" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM17" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN17" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO17" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP17" s="5" t="inlineStr">
@@ -3719,35 +3719,35 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>23336013</v>
+        <v>24507740</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>24064303</v>
+        <v>25321974</v>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>ACC04</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
-        <v>45977.77516203704</v>
+        <v>46139.78204861111</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>45979.38710648148</v>
+        <v>46139.78418981482</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>GMKD4Q</t>
+          <t>MWEAPK</t>
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr">
@@ -3757,7 +3757,7 @@
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Rafael Vieira</t>
+          <t>Cleizer Bessa</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -3771,10 +3771,10 @@
         </is>
       </c>
       <c r="M18" s="6" t="n">
-        <v>45977.77430555555</v>
+        <v>46139.78125</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>6954279</v>
+        <v>7370194</v>
       </c>
       <c r="O18" s="5" t="inlineStr">
         <is>
@@ -3803,7 +3803,7 @@
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
@@ -3813,7 +3813,7 @@
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Cleizer</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -3823,11 +3823,11 @@
       </c>
       <c r="X18" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y18" s="5" t="n">
-        <v>2846058807</v>
+        <v>2284371064</v>
       </c>
       <c r="Z18" s="5" t="inlineStr">
         <is>
@@ -3840,10 +3840,10 @@
         </is>
       </c>
       <c r="AB18" s="5" t="n">
-        <v>0</v>
+        <v>554.72</v>
       </c>
       <c r="AC18" s="5" t="n">
-        <v>0</v>
+        <v>34.11</v>
       </c>
       <c r="AD18" s="5" t="n">
         <v>0</v>
@@ -3858,7 +3858,7 @@
         <v>0</v>
       </c>
       <c r="AH18" s="5" t="n">
-        <v>0</v>
+        <v>135.14</v>
       </c>
       <c r="AI18" s="5" t="inlineStr">
         <is>
@@ -3867,7 +3867,7 @@
       </c>
       <c r="AJ18" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK18" s="5" t="inlineStr">
@@ -3877,22 +3877,22 @@
       </c>
       <c r="AL18" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM18" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN18" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO18" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP18" s="5" t="inlineStr">
@@ -3908,35 +3908,35 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>23336013</v>
+        <v>24507740</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>24064304</v>
+        <v>25321976</v>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>ACC05</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
-        <v>45977.77516203704</v>
+        <v>46139.78204861111</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>45979.38710648148</v>
+        <v>46139.78418981482</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>GMKD4Q</t>
+          <t>MWEAPK</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
@@ -3946,7 +3946,7 @@
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Luisa Delgado</t>
+          <t>Carlos Santos</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -3960,10 +3960,10 @@
         </is>
       </c>
       <c r="M19" s="6" t="n">
-        <v>45977.77430555555</v>
+        <v>46139.78125</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>6954279</v>
+        <v>7370194</v>
       </c>
       <c r="O19" s="5" t="inlineStr">
         <is>
@@ -3992,7 +3992,7 @@
       </c>
       <c r="T19" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U19" s="5" t="inlineStr">
@@ -4002,7 +4002,7 @@
       </c>
       <c r="V19" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Cleizer</t>
         </is>
       </c>
       <c r="W19" s="5" t="inlineStr">
@@ -4012,11 +4012,11 @@
       </c>
       <c r="X19" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
+          <t>Latam Airlines Brasil</t>
         </is>
       </c>
       <c r="Y19" s="5" t="n">
-        <v>2252583666</v>
+        <v>2284371065</v>
       </c>
       <c r="Z19" s="5" t="inlineStr">
         <is>
@@ -4029,10 +4029,10 @@
         </is>
       </c>
       <c r="AB19" s="5" t="n">
-        <v>0</v>
+        <v>554.72</v>
       </c>
       <c r="AC19" s="5" t="n">
-        <v>0</v>
+        <v>34.11</v>
       </c>
       <c r="AD19" s="5" t="n">
         <v>0</v>
@@ -4056,7 +4056,7 @@
       </c>
       <c r="AJ19" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395430. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK19" s="5" t="inlineStr">
@@ -4066,22 +4066,22 @@
       </c>
       <c r="AL19" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM19" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN19" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO19" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP19" s="5" t="inlineStr">
@@ -4097,10 +4097,10 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="n">
-        <v>23336052</v>
+        <v>24505190</v>
       </c>
       <c r="B20" s="5" t="n">
-        <v>24064343</v>
+        <v>25319047</v>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
@@ -4108,34 +4108,32 @@
         </is>
       </c>
       <c r="D20" s="6" t="n">
-        <v>45977.7834375</v>
+        <v>46139.52736111111</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>45979.38715277778</v>
+        <v>46139.52982638889</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>BL8JGG</t>
-        </is>
+          <t>0 a 02 dias</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>15241774</v>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>EBOOKING</t>
+          <t>MANUAL</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Giullia Delgado</t>
+          <t>ROMEU GOMES MELO</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -4149,10 +4147,12 @@
         </is>
       </c>
       <c r="M20" s="6" t="n">
-        <v>45977.78263888889</v>
-      </c>
-      <c r="N20" s="5" t="n">
-        <v>6954301</v>
+        <v>46138.41666666666</v>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="O20" s="5" t="inlineStr">
         <is>
@@ -4176,12 +4176,12 @@
       </c>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Aéreo</t>
+          <t>Serviço</t>
         </is>
       </c>
       <c r="T20" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U20" s="5" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="V20" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Romeu Gomes Melo</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -4201,11 +4201,13 @@
       </c>
       <c r="X20" s="5" t="inlineStr">
         <is>
-          <t>Azul Linhas Aereas</t>
-        </is>
-      </c>
-      <c r="Y20" s="5" t="n">
-        <v>3340742969</v>
+          <t>Universal Assistance</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="Z20" s="5" t="inlineStr">
         <is>
@@ -4218,10 +4220,10 @@
         </is>
       </c>
       <c r="AB20" s="5" t="n">
-        <v>404.38</v>
+        <v>40.5</v>
       </c>
       <c r="AC20" s="5" t="n">
-        <v>58.89</v>
+        <v>0</v>
       </c>
       <c r="AD20" s="5" t="n">
         <v>0</v>
@@ -4236,16 +4238,16 @@
         <v>0</v>
       </c>
       <c r="AH20" s="5" t="n">
-        <v>151.32</v>
+        <v>0</v>
       </c>
       <c r="AI20" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Seguro Viagem</t>
         </is>
       </c>
       <c r="AJ20" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK20" s="5" t="inlineStr">
@@ -4255,22 +4257,22 @@
       </c>
       <c r="AL20" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM20" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN20" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO20" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP20" s="5" t="inlineStr">
@@ -4286,10 +4288,10 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>23336392</v>
+        <v>24506625</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>24064696</v>
+        <v>25320672</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
@@ -4297,24 +4299,24 @@
         </is>
       </c>
       <c r="D21" s="6" t="n">
-        <v>45977.85212962963</v>
+        <v>46139.6521412037</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>45979.38746527778</v>
+        <v>46139.6528125</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>MJ7MKP</t>
+          <t>GM9VNG</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
@@ -4324,7 +4326,7 @@
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Jose Figueiredo</t>
+          <t>Cleizer Bessa</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -4338,10 +4340,10 @@
         </is>
       </c>
       <c r="M21" s="6" t="n">
-        <v>45977.85138888889</v>
+        <v>46139.65138888889</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>6954464</v>
+        <v>7369680</v>
       </c>
       <c r="O21" s="5" t="inlineStr">
         <is>
@@ -4370,7 +4372,7 @@
       </c>
       <c r="T21" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U21" s="5" t="inlineStr">
@@ -4380,7 +4382,7 @@
       </c>
       <c r="V21" s="5" t="inlineStr">
         <is>
-          <t>Jose Antonio de Figueiredo</t>
+          <t>Cleizer</t>
         </is>
       </c>
       <c r="W21" s="5" t="inlineStr">
@@ -4394,7 +4396,7 @@
         </is>
       </c>
       <c r="Y21" s="5" t="n">
-        <v>9825033326</v>
+        <v>5302655319</v>
       </c>
       <c r="Z21" s="5" t="inlineStr">
         <is>
@@ -4407,10 +4409,10 @@
         </is>
       </c>
       <c r="AB21" s="5" t="n">
-        <v>1662.64</v>
+        <v>930.62</v>
       </c>
       <c r="AC21" s="5" t="n">
-        <v>39.58</v>
+        <v>52.72</v>
       </c>
       <c r="AD21" s="5" t="n">
         <v>0</v>
@@ -4425,7 +4427,7 @@
         <v>0</v>
       </c>
       <c r="AH21" s="5" t="n">
-        <v>405.68</v>
+        <v>113.06</v>
       </c>
       <c r="AI21" s="5" t="inlineStr">
         <is>
@@ -4434,7 +4436,7 @@
       </c>
       <c r="AJ21" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395732. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK21" s="5" t="inlineStr">
@@ -4444,22 +4446,22 @@
       </c>
       <c r="AL21" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM21" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN21" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO21" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP21" s="5" t="inlineStr">
@@ -4475,10 +4477,10 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
-        <v>23336392</v>
+        <v>24506625</v>
       </c>
       <c r="B22" s="5" t="n">
-        <v>24064697</v>
+        <v>25320673</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
@@ -4486,24 +4488,24 @@
         </is>
       </c>
       <c r="D22" s="6" t="n">
-        <v>45977.85212962963</v>
+        <v>46139.6521412037</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>45979.38746527778</v>
+        <v>46139.6528125</v>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>MJ7MKP</t>
+          <t>GM9VNG</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
@@ -4513,7 +4515,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Kelmey Santos</t>
+          <t>Carlos Henrique Santos</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -4527,10 +4529,10 @@
         </is>
       </c>
       <c r="M22" s="6" t="n">
-        <v>45977.85138888889</v>
+        <v>46139.65138888889</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>6954464</v>
+        <v>7369680</v>
       </c>
       <c r="O22" s="5" t="inlineStr">
         <is>
@@ -4559,7 +4561,7 @@
       </c>
       <c r="T22" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
@@ -4569,7 +4571,7 @@
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>Jose Antonio de Figueiredo</t>
+          <t>Cleizer</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -4583,7 +4585,7 @@
         </is>
       </c>
       <c r="Y22" s="5" t="n">
-        <v>1720811985</v>
+        <v>8235628381</v>
       </c>
       <c r="Z22" s="5" t="inlineStr">
         <is>
@@ -4596,10 +4598,10 @@
         </is>
       </c>
       <c r="AB22" s="5" t="n">
-        <v>1662.64</v>
+        <v>930.62</v>
       </c>
       <c r="AC22" s="5" t="n">
-        <v>39.58</v>
+        <v>52.72</v>
       </c>
       <c r="AD22" s="5" t="n">
         <v>0</v>
@@ -4623,7 +4625,7 @@
       </c>
       <c r="AJ22" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395732. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK22" s="5" t="inlineStr">
@@ -4633,22 +4635,22 @@
       </c>
       <c r="AL22" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM22" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN22" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO22" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP22" s="5" t="inlineStr">
@@ -4664,35 +4666,35 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>23336052</v>
+        <v>24507731</v>
       </c>
       <c r="B23" s="5" t="n">
-        <v>24064346</v>
+        <v>25321962</v>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>ACC04</t>
+          <t>ACC01</t>
         </is>
       </c>
       <c r="D23" s="6" t="n">
-        <v>45977.7834375</v>
+        <v>46139.78134259259</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>45979.38715277778</v>
+        <v>46139.78228009259</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>BL8JGG</t>
+          <t>BPP87H</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
@@ -4702,7 +4704,7 @@
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Rafael Vieira</t>
+          <t>Cleizer Bessa</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -4716,10 +4718,10 @@
         </is>
       </c>
       <c r="M23" s="6" t="n">
-        <v>45977.78263888889</v>
+        <v>46139.78055555555</v>
       </c>
       <c r="N23" s="5" t="n">
-        <v>6954301</v>
+        <v>7370192</v>
       </c>
       <c r="O23" s="5" t="inlineStr">
         <is>
@@ -4748,7 +4750,7 @@
       </c>
       <c r="T23" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U23" s="5" t="inlineStr">
@@ -4758,7 +4760,7 @@
       </c>
       <c r="V23" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Cleizer</t>
         </is>
       </c>
       <c r="W23" s="5" t="inlineStr">
@@ -4772,7 +4774,7 @@
         </is>
       </c>
       <c r="Y23" s="5" t="n">
-        <v>4961395002</v>
+        <v>8154303333</v>
       </c>
       <c r="Z23" s="5" t="inlineStr">
         <is>
@@ -4785,10 +4787,10 @@
         </is>
       </c>
       <c r="AB23" s="5" t="n">
-        <v>0</v>
+        <v>1134.9</v>
       </c>
       <c r="AC23" s="5" t="n">
-        <v>0</v>
+        <v>52.72</v>
       </c>
       <c r="AD23" s="5" t="n">
         <v>0</v>
@@ -4803,7 +4805,7 @@
         <v>0</v>
       </c>
       <c r="AH23" s="5" t="n">
-        <v>0</v>
+        <v>136.18</v>
       </c>
       <c r="AI23" s="5" t="inlineStr">
         <is>
@@ -4812,7 +4814,7 @@
       </c>
       <c r="AJ23" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK23" s="5" t="inlineStr">
@@ -4822,22 +4824,22 @@
       </c>
       <c r="AL23" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM23" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN23" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO23" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP23" s="5" t="inlineStr">
@@ -4853,35 +4855,35 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
-        <v>23336052</v>
+        <v>24507731</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>24064347</v>
+        <v>25321965</v>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>ACC05</t>
+          <t>ACC02</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>45977.7834375</v>
+        <v>46139.78134259259</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>45979.38715277778</v>
+        <v>46139.78228009259</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>06 a 08 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>09 a 15 dias</t>
+          <t>0 a 02 dias</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>BL8JGG</t>
+          <t>BPP87H</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
@@ -4891,7 +4893,7 @@
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Luisa Delgado</t>
+          <t>Carlos Santos</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -4905,10 +4907,10 @@
         </is>
       </c>
       <c r="M24" s="6" t="n">
-        <v>45977.78263888889</v>
+        <v>46139.78055555555</v>
       </c>
       <c r="N24" s="5" t="n">
-        <v>6954301</v>
+        <v>7370192</v>
       </c>
       <c r="O24" s="5" t="inlineStr">
         <is>
@@ -4937,7 +4939,7 @@
       </c>
       <c r="T24" s="5" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="U24" s="5" t="inlineStr">
@@ -4947,7 +4949,7 @@
       </c>
       <c r="V24" s="5" t="inlineStr">
         <is>
-          <t>Giulianna Angelica Piason de Brito</t>
+          <t>Cleizer</t>
         </is>
       </c>
       <c r="W24" s="5" t="inlineStr">
@@ -4961,7 +4963,7 @@
         </is>
       </c>
       <c r="Y24" s="5" t="n">
-        <v>2175324568</v>
+        <v>1800262606</v>
       </c>
       <c r="Z24" s="5" t="inlineStr">
         <is>
@@ -4974,10 +4976,10 @@
         </is>
       </c>
       <c r="AB24" s="5" t="n">
-        <v>0</v>
+        <v>1134.9</v>
       </c>
       <c r="AC24" s="5" t="n">
-        <v>0</v>
+        <v>52.72</v>
       </c>
       <c r="AD24" s="5" t="n">
         <v>0</v>
@@ -5001,7 +5003,7 @@
       </c>
       <c r="AJ24" s="5" t="inlineStr">
         <is>
-          <t>Erro excluindo PNR: Não é possivel excluir a accounting de código: 25395461. A mesma está ligada a conciliação de cartão "PAYMEE 17.11.2025.xlsx"</t>
+          <t>Não foi possível definir o Local de destino!</t>
         </is>
       </c>
       <c r="AK24" s="5" t="inlineStr">
@@ -5011,22 +5013,22 @@
       </c>
       <c r="AL24" s="5" t="inlineStr">
         <is>
-          <t>Conciliação de Cartão</t>
+          <t>Cadastro enviado errado no Benner</t>
         </is>
       </c>
       <c r="AM24" s="5" t="inlineStr">
         <is>
-          <t>Financeiro Conciliado</t>
+          <t>Cadastro incompleto</t>
         </is>
       </c>
       <c r="AN24" s="5" t="inlineStr">
         <is>
-          <t>Edição não Permitida</t>
+          <t>Sistema</t>
         </is>
       </c>
       <c r="AO24" s="5" t="inlineStr">
         <is>
-          <t>Processo Operacional</t>
+          <t>Sistêmico</t>
         </is>
       </c>
       <c r="AP24" s="5" t="inlineStr">
@@ -5035,6 +5037,195 @@
         </is>
       </c>
       <c r="AQ24" s="5" t="inlineStr">
+        <is>
+          <t>Operações - ZUPPER</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>24505371</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>25319250</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>ACC01</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>46139.55082175926</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>46139.55329861111</v>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>0 a 02 dias</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>0 a 02 dias</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>XNBYJG</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>EBOOKING</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>Anderson Mello</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Zupper</t>
+        </is>
+      </c>
+      <c r="M25" s="6" t="n">
+        <v>46139.55</v>
+      </c>
+      <c r="N25" s="5" t="n">
+        <v>7369315</v>
+      </c>
+      <c r="O25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P25" s="5" t="inlineStr">
+        <is>
+          <t>OFF LINE</t>
+        </is>
+      </c>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>Cartão convênio</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>Aéreo</t>
+        </is>
+      </c>
+      <c r="T25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U25" s="5" t="inlineStr">
+        <is>
+          <t>Grupo Zupper</t>
+        </is>
+      </c>
+      <c r="V25" s="5" t="inlineStr">
+        <is>
+          <t>Anderson Marcelo Mello</t>
+        </is>
+      </c>
+      <c r="W25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X25" s="5" t="inlineStr">
+        <is>
+          <t>Azul Linhas Aereas</t>
+        </is>
+      </c>
+      <c r="Y25" s="5" t="n">
+        <v>3155460315</v>
+      </c>
+      <c r="Z25" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AA25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB25" s="5" t="n">
+        <v>671.51</v>
+      </c>
+      <c r="AC25" s="5" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="AD25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH25" s="5" t="n">
+        <v>43.58</v>
+      </c>
+      <c r="AI25" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AJ25" s="5" t="inlineStr">
+        <is>
+          <t>Não foi possível definir o Local de destino!</t>
+        </is>
+      </c>
+      <c r="AK25" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER</t>
+        </is>
+      </c>
+      <c r="AL25" s="5" t="inlineStr">
+        <is>
+          <t>Cadastro enviado errado no Benner</t>
+        </is>
+      </c>
+      <c r="AM25" s="5" t="inlineStr">
+        <is>
+          <t>Cadastro incompleto</t>
+        </is>
+      </c>
+      <c r="AN25" s="5" t="inlineStr">
+        <is>
+          <t>Sistema</t>
+        </is>
+      </c>
+      <c r="AO25" s="5" t="inlineStr">
+        <is>
+          <t>Sistêmico</t>
+        </is>
+      </c>
+      <c r="AP25" s="5" t="inlineStr">
+        <is>
+          <t>ZUPPER VIAGENS</t>
+        </is>
+      </c>
+      <c r="AQ25" s="5" t="inlineStr">
         <is>
           <t>Operações - ZUPPER</t>
         </is>

</xml_diff>